<commit_message>
otimização no tempo de busca
</commit_message>
<xml_diff>
--- a/relatorio_rpv.xlsx
+++ b/relatorio_rpv.xlsx
@@ -486,13 +486,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
     <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="3" max="3"/>
+    <col width="23" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -531,7 +531,7 @@
       <c r="C2" s="5" t="inlineStr"/>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>RPV4357095-PE</t>
+          <t>2026830002016500799</t>
         </is>
       </c>
     </row>
@@ -553,7 +553,7 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>RPV4348849-CE</t>
+          <t>2026810000020500360</t>
         </is>
       </c>
     </row>
@@ -575,19 +575,19 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>RPV4348838-CE</t>
+          <t>2026810000020500364</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>0459910-03.2026.4.05.0000</t>
+          <t>0452226-27.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>20º VF CE</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
@@ -597,19 +597,19 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>RPV4348832-CE</t>
+          <t>2026800000014508334</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>0452226-27.2026.4.05.0000</t>
+          <t>0448842-56.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>20º VF CE</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -619,19 +619,19 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>RPV4341264-AL</t>
+          <t>2026810000020500407</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>0451693-68.2026.4.05.0000</t>
+          <t>0448852-03.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>20º VF CE</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -641,7 +641,7 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>RPV4340731-AL</t>
+          <t>2026810000020500409</t>
         </is>
       </c>
     </row>
@@ -663,14 +663,14 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>RPV4337946-CE</t>
+          <t>2026810000020500411</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>0448842-56.2026.4.05.0000</t>
+          <t>0459910-03.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
@@ -685,19 +685,19 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>RPV4337940-CE</t>
+          <t>2026810000020500361</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>0448852-03.2026.4.05.0000</t>
+          <t>0451693-68.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>20º VF CE</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -707,7 +707,7 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>RPV4337950-CE</t>
+          <t>2026800000014507677</t>
         </is>
       </c>
     </row>
@@ -729,7 +729,1947 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>RPV4334816-RN</t>
+          <t>2026840000007506232</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>0443066-75.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>20º VF CE</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>2026810000020500391</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>0422526-06.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>7º VF RN</t>
+        </is>
+      </c>
+      <c r="C13" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>2026840000007504848</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>0440333-39.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>33º VF CE</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>2026810000033500155</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>0434796-62.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>33º VF CE</t>
+        </is>
+      </c>
+      <c r="C15" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D15" s="7" t="inlineStr">
+        <is>
+          <t>2026810000033500132</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>0433722-70.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="inlineStr">
+        <is>
+          <t>20º VF CE</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="inlineStr">
+        <is>
+          <t>2026810000020500262</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>0440075-29.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>20º VF CE</t>
+        </is>
+      </c>
+      <c r="C17" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>2026810000020500345</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>0443063-23.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>20º VF CE</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D18" s="4" t="inlineStr">
+        <is>
+          <t>2026810000020500388</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>0440332-54.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>33º VF CE</t>
+        </is>
+      </c>
+      <c r="C19" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D19" s="7" t="inlineStr">
+        <is>
+          <t>2026810000033500154</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>0440886-86.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>4º VF SE</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D20" s="4" t="inlineStr">
+        <is>
+          <t>2026850000004500380</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>0432087-54.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>33º VF CE</t>
+        </is>
+      </c>
+      <c r="C21" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D21" s="7" t="inlineStr">
+        <is>
+          <t>2026810000033500131</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>0421015-70.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>9º VF PE</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D22" s="4" t="inlineStr">
+        <is>
+          <t>2026840002009501445</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>0432115-22.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C23" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D23" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006508048</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>0429599-29.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>2026800000009504071</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>0429600-14.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C25" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D25" s="7" t="inlineStr">
+        <is>
+          <t>2026800000009504072</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>0432006-08.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>11º VF AL</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D26" s="4" t="inlineStr">
+        <is>
+          <t>2026800003011505673</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="6" t="inlineStr">
+        <is>
+          <t>0429605-36.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C27" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D27" s="7" t="inlineStr">
+        <is>
+          <t>2026800000009504043</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>0433003-88.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>4º VF SE</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>2026850000004500263</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="6" t="inlineStr">
+        <is>
+          <t>0429807-13.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D29" s="7" t="inlineStr">
+        <is>
+          <t>2026800000009504294</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>0421013-03.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>9º VF PE</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>2026840002009501374</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="6" t="inlineStr">
+        <is>
+          <t>0432271-10.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>1º VF PB</t>
+        </is>
+      </c>
+      <c r="C31" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D31" s="7" t="inlineStr">
+        <is>
+          <t>2026820000001500268</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>0435911-21.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>3º VF PE</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D32" s="4" t="inlineStr">
+        <is>
+          <t>2026850000003500131</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>0436433-48.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C33" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D33" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006508281</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>0440400-04.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>25º VF PE</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D34" s="4" t="inlineStr">
+        <is>
+          <t>2026830006025502135</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="6" t="inlineStr">
+        <is>
+          <t>0442485-60.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>14º VF PE</t>
+        </is>
+      </c>
+      <c r="C35" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D35" s="7" t="inlineStr">
+        <is>
+          <t>2026830000014503418</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>0445330-65.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D36" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006508563</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="6" t="inlineStr">
+        <is>
+          <t>0439583-37.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>12º VF AL</t>
+        </is>
+      </c>
+      <c r="C37" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D37" s="7" t="inlineStr">
+        <is>
+          <t>2026800001012503362</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>0439844-02.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D38" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006508482</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>0436398-88.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C39" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006508316</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>0444257-58.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B40" s="4" t="inlineStr">
+        <is>
+          <t>9º VF CE</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D40" s="4" t="inlineStr">
+        <is>
+          <t>2026810000009500096</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>0440202-64.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>19º VF PE</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>2026830000019502593</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>0445352-26.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B42" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D42" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006508585</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>0445358-33.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006508591</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>0445489-08.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B44" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D44" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006508650</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>0451653-86.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C45" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>2026800000014507587</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>0447817-08.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B46" s="4" t="inlineStr">
+        <is>
+          <t>9º VF PB</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D46" s="4" t="inlineStr">
+        <is>
+          <t>2026820001009502477</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>0445470-02.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006508699</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>0451459-86.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B48" s="4" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D48" s="4" t="inlineStr">
+        <is>
+          <t>2026800000014507369</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>0450523-61.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>2026800000014506466</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>0450167-66.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B50" s="4" t="inlineStr">
+        <is>
+          <t>14º VF PE</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D50" s="4" t="inlineStr">
+        <is>
+          <t>2026830000014503061</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>0448213-82.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>2026800000009503783</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>0451747-34.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B52" s="4" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D52" s="4" t="inlineStr">
+        <is>
+          <t>2026800000014507488</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>0452536-33.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>2026800000014508690</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>0452009-81.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B54" s="4" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="inlineStr">
+        <is>
+          <t>2026800000014508108</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>0452256-62.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>2026800000014506443</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>0452601-28.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B56" s="4" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D56" s="4" t="inlineStr">
+        <is>
+          <t>2026800000014508618</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>0452854-16.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>2026800000014508192</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>0452384-82.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C58" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>2026800000014507635</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>0452501-73.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>2026800000014508173</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>0452306-88.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B60" s="4" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D60" s="4" t="inlineStr">
+        <is>
+          <t>2026800000014508366</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>0452735-55.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D61" s="7" t="inlineStr">
+        <is>
+          <t>2026800000014508926</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>0454207-91.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B62" s="4" t="inlineStr">
+        <is>
+          <t>7º VF RN</t>
+        </is>
+      </c>
+      <c r="C62" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D62" s="4" t="inlineStr">
+        <is>
+          <t>2026840000007505433</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>0422323-44.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>7º VF RN</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D63" s="7" t="inlineStr">
+        <is>
+          <t>2026840000007503056</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>0459281-29.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B64" s="4" t="inlineStr">
+        <is>
+          <t>14º VF PE</t>
+        </is>
+      </c>
+      <c r="C64" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D64" s="4" t="inlineStr">
+        <is>
+          <t>2026830000014504238</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>0426515-20.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D65" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006507810</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>0459836-46.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B66" s="4" t="inlineStr">
+        <is>
+          <t>3º VF RN</t>
+        </is>
+      </c>
+      <c r="C66" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D66" s="4" t="inlineStr">
+        <is>
+          <t>2026840000003503607</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>0461413-59.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>34º VF PE</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D67" s="7" t="inlineStr">
+        <is>
+          <t>2026830012034500718</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>0423263-09.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B68" s="4" t="inlineStr">
+        <is>
+          <t>7º VF RN</t>
+        </is>
+      </c>
+      <c r="C68" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>2026840000007505332</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>0458573-76.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>13º VF PE</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D69" s="7" t="inlineStr">
+        <is>
+          <t>2026820000013510143</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="22" customHeight="1">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>0458903-73.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B70" s="4" t="inlineStr">
+        <is>
+          <t>3º VF PE</t>
+        </is>
+      </c>
+      <c r="C70" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>2026820000003500707</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="22" customHeight="1">
+      <c r="A71" s="6" t="inlineStr">
+        <is>
+          <t>0422322-59.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B71" s="7" t="inlineStr">
+        <is>
+          <t>7º VF RN</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D71" s="7" t="inlineStr">
+        <is>
+          <t>2026840000007503047</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="22" customHeight="1">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>0426615-72.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B72" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C72" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006507954</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="22" customHeight="1">
+      <c r="A73" s="6" t="inlineStr">
+        <is>
+          <t>0429144-64.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B73" s="7" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D73" s="7" t="inlineStr">
+        <is>
+          <t>2026800000009503319</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="22" customHeight="1">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>0426618-27.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B74" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006507957</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="22" customHeight="1">
+      <c r="A75" s="6" t="inlineStr">
+        <is>
+          <t>0429070-10.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B75" s="7" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D75" s="7" t="inlineStr">
+        <is>
+          <t>2026800000009503137</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="22" customHeight="1">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>0428095-85.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B76" s="4" t="inlineStr">
+        <is>
+          <t>10º VF AL</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>2026800001010503452</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="22" customHeight="1">
+      <c r="A77" s="6" t="inlineStr">
+        <is>
+          <t>0426978-59.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B77" s="7" t="inlineStr">
+        <is>
+          <t>11º VF AL</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D77" s="7" t="inlineStr">
+        <is>
+          <t>2026800003011505648</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="22" customHeight="1">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>0427483-50.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B78" s="4" t="inlineStr">
+        <is>
+          <t>30º VF PE</t>
+        </is>
+      </c>
+      <c r="C78" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>2026830011030502090</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="22" customHeight="1">
+      <c r="A79" s="6" t="inlineStr">
+        <is>
+          <t>0429143-79.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B79" s="7" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C79" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D79" s="7" t="inlineStr">
+        <is>
+          <t>2026800000009503318</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="22" customHeight="1">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>0429031-13.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B80" s="4" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>2026800000009502988</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="22" customHeight="1">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>0428241-29.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>13º VF AL</t>
+        </is>
+      </c>
+      <c r="C81" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D81" s="7" t="inlineStr">
+        <is>
+          <t>2026800000013500090</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" ht="22" customHeight="1">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>0429381-98.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B82" s="4" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>2026800000009503562</t>
+        </is>
+      </c>
+    </row>
+    <row r="83" ht="22" customHeight="1">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>0429395-82.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C83" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D83" s="7" t="inlineStr">
+        <is>
+          <t>2026800000009503544</t>
+        </is>
+      </c>
+    </row>
+    <row r="84" ht="22" customHeight="1">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>0464899-52.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B84" s="4" t="inlineStr">
+        <is>
+          <t>14º VF PE</t>
+        </is>
+      </c>
+      <c r="C84" s="5" t="inlineStr"/>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>2026830000014504627</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" ht="22" customHeight="1">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>0466785-86.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>7º VF AL</t>
+        </is>
+      </c>
+      <c r="C85" s="8" t="inlineStr"/>
+      <c r="D85" s="7" t="inlineStr">
+        <is>
+          <t>2026800002007503620</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" ht="22" customHeight="1">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>0429598-44.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B86" s="4" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>2026800000009504069</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="22" customHeight="1">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>0464849-26.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>7º VF RN</t>
+        </is>
+      </c>
+      <c r="C87" s="8" t="inlineStr"/>
+      <c r="D87" s="7" t="inlineStr">
+        <is>
+          <t>2026840000007505544</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="22" customHeight="1">
+      <c r="A88" s="3" t="inlineStr">
+        <is>
+          <t>0464331-36.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C88" s="5" t="inlineStr"/>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006509055</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="22" customHeight="1">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>0464605-97.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="inlineStr"/>
+      <c r="D89" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006509381</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="22" customHeight="1">
+      <c r="A90" s="3" t="inlineStr">
+        <is>
+          <t>0429596-74.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>2026800000009504063</t>
+        </is>
+      </c>
+    </row>
+    <row r="91" ht="22" customHeight="1">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>0464356-49.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C91" s="8" t="inlineStr"/>
+      <c r="D91" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006509082</t>
+        </is>
+      </c>
+    </row>
+    <row r="92" ht="22" customHeight="1">
+      <c r="A92" s="3" t="inlineStr">
+        <is>
+          <t>0464329-66.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B92" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr"/>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006509053</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="22" customHeight="1">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>0461673-39.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>30º VF PE</t>
+        </is>
+      </c>
+      <c r="C93" s="8" t="inlineStr"/>
+      <c r="D93" s="7" t="inlineStr">
+        <is>
+          <t>2026830011030502351</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="22" customHeight="1">
+      <c r="A94" s="3" t="inlineStr">
+        <is>
+          <t>0418861-79.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B94" s="4" t="inlineStr">
+        <is>
+          <t>10º VF AL</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>2026800001010502803</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="22" customHeight="1">
+      <c r="A95" s="6" t="inlineStr">
+        <is>
+          <t>0419484-46.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>10º VF AL</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D95" s="7" t="inlineStr">
+        <is>
+          <t>2026800001010503210</t>
+        </is>
+      </c>
+    </row>
+    <row r="96" ht="22" customHeight="1">
+      <c r="A96" s="3" t="inlineStr">
+        <is>
+          <t>0461780-83.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B96" s="4" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C96" s="5" t="inlineStr"/>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>2026800000009504875</t>
+        </is>
+      </c>
+    </row>
+    <row r="97" ht="22" customHeight="1">
+      <c r="A97" s="6" t="inlineStr">
+        <is>
+          <t>0401993-26.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B97" s="7" t="inlineStr">
+        <is>
+          <t>2º VF PE</t>
+        </is>
+      </c>
+      <c r="C97" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D97" s="7" t="inlineStr">
+        <is>
+          <t>2026830000002500220</t>
+        </is>
+      </c>
+    </row>
+    <row r="98" ht="22" customHeight="1">
+      <c r="A98" s="3" t="inlineStr">
+        <is>
+          <t>0464221-37.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B98" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C98" s="5" t="inlineStr"/>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006508945</t>
+        </is>
+      </c>
+    </row>
+    <row r="99" ht="22" customHeight="1">
+      <c r="A99" s="6" t="inlineStr">
+        <is>
+          <t>0411960-95.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B99" s="7" t="inlineStr">
+        <is>
+          <t>20º VF CE</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D99" s="7" t="inlineStr">
+        <is>
+          <t>2026810000020500292</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="22" customHeight="1">
+      <c r="A100" s="3" t="inlineStr">
+        <is>
+          <t>0393292-76.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>2º VF SE</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>2026850000002500075</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="22" customHeight="1">
+      <c r="A101" s="6" t="inlineStr">
+        <is>
+          <t>0397570-23.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B101" s="7" t="inlineStr">
+        <is>
+          <t>4º VF SE</t>
+        </is>
+      </c>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D101" s="7" t="inlineStr">
+        <is>
+          <t>2026850000004500323</t>
         </is>
       </c>
     </row>
@@ -745,6 +2685,96 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId8"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId9"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A26" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A27" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A28" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A29" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A30" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A31" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A32" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A33" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A34" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A35" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A36" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A37" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A38" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A39" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A40" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A41" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A42" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A43" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A44" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A45" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A46" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A47" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A48" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A49" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A50" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A51" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A52" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A53" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A54" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A55" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A56" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A57" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A58" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A59" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A60" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A101" r:id="rId100"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Versao segura do sistema
</commit_message>
<xml_diff>
--- a/relatorio_rpv.xlsx
+++ b/relatorio_rpv.xlsx
@@ -486,7 +486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D101"/>
+  <dimension ref="A1:D201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="29" customWidth="1" min="1" max="1"/>
@@ -520,30 +520,34 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>0468287-60.2026.4.05.0000</t>
+          <t>0458903-73.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>16º VF PE</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr"/>
+          <t>3º VF PE</t>
+        </is>
+      </c>
+      <c r="C2" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>2026830002016500799</t>
+          <t>2026820000003500707</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>0459927-39.2026.4.05.0000</t>
+          <t>0452735-55.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
         <is>
-          <t>20º VF CE</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -553,19 +557,19 @@
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>2026810000020500360</t>
+          <t>2026800000014508926</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>0459916-10.2026.4.05.0000</t>
+          <t>0459281-29.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>20º VF CE</t>
+          <t>14º VF PE</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
@@ -575,14 +579,14 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>2026810000020500364</t>
+          <t>2026830000014504238</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>0452226-27.2026.4.05.0000</t>
+          <t>0452601-28.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B5" s="7" t="inlineStr">
@@ -597,19 +601,19 @@
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>2026800000014508334</t>
+          <t>2026800000014508618</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>0448842-56.2026.4.05.0000</t>
+          <t>0452501-73.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>20º VF CE</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="C6" s="5" t="inlineStr">
@@ -619,19 +623,19 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>2026810000020500407</t>
+          <t>2026800000014508173</t>
         </is>
       </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>0448852-03.2026.4.05.0000</t>
+          <t>0458573-76.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B7" s="7" t="inlineStr">
         <is>
-          <t>20º VF CE</t>
+          <t>13º VF PE</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
@@ -641,19 +645,19 @@
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
-          <t>2026810000020500409</t>
+          <t>2026820000013510143</t>
         </is>
       </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>0448848-63.2026.4.05.0000</t>
+          <t>0452536-33.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>20º VF CE</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="C8" s="5" t="inlineStr">
@@ -663,19 +667,19 @@
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>2026810000020500411</t>
+          <t>2026800000014508690</t>
         </is>
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>0459910-03.2026.4.05.0000</t>
+          <t>0452854-16.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B9" s="7" t="inlineStr">
         <is>
-          <t>20º VF CE</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="C9" s="8" t="inlineStr">
@@ -685,19 +689,19 @@
       </c>
       <c r="D9" s="7" t="inlineStr">
         <is>
-          <t>2026810000020500361</t>
+          <t>2026800000014508192</t>
         </is>
       </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>0451693-68.2026.4.05.0000</t>
+          <t>0454207-91.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>7º VF RN</t>
         </is>
       </c>
       <c r="C10" s="5" t="inlineStr">
@@ -707,19 +711,19 @@
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>2026800000014507677</t>
+          <t>2026840000007505433</t>
         </is>
       </c>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>0445686-60.2026.4.05.0000</t>
+          <t>0452384-82.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B11" s="7" t="inlineStr">
         <is>
-          <t>7º VF RN</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="C11" s="8" t="inlineStr">
@@ -729,19 +733,19 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>2026840000007506232</t>
+          <t>2026800000014507635</t>
         </is>
       </c>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>0443066-75.2026.4.05.0000</t>
+          <t>0452306-88.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>20º VF CE</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
@@ -751,41 +755,41 @@
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>2026810000020500391</t>
+          <t>2026800000014508366</t>
         </is>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>0422526-06.2026.4.05.0000</t>
+          <t>0451653-86.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B13" s="7" t="inlineStr">
         <is>
-          <t>7º VF RN</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="C13" s="8" t="inlineStr">
         <is>
-          <t>Caixa Econômica Federal</t>
+          <t>Banco do Brasil S/A</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
         <is>
-          <t>2026840000007504848</t>
+          <t>2026800000014507587</t>
         </is>
       </c>
     </row>
     <row r="14" ht="22" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>0440333-39.2026.4.05.0000</t>
+          <t>0451747-34.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>33º VF CE</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
@@ -795,63 +799,63 @@
       </c>
       <c r="D14" s="4" t="inlineStr">
         <is>
-          <t>2026810000033500155</t>
+          <t>2026800000014507488</t>
         </is>
       </c>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>0434796-62.2026.4.05.0000</t>
+          <t>0451693-68.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B15" s="7" t="inlineStr">
         <is>
-          <t>33º VF CE</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="C15" s="8" t="inlineStr">
         <is>
-          <t>Caixa Econômica Federal</t>
+          <t>Banco do Brasil S/A</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
         <is>
-          <t>2026810000033500132</t>
+          <t>2026800000014507677</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>0433722-70.2026.4.05.0000</t>
+          <t>0452256-62.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>20º VF CE</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>Caixa Econômica Federal</t>
+          <t>Banco do Brasil S/A</t>
         </is>
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>2026810000020500262</t>
+          <t>2026800000014506443</t>
         </is>
       </c>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>0440075-29.2026.4.05.0000</t>
+          <t>0450167-66.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>20º VF CE</t>
+          <t>14º VF PE</t>
         </is>
       </c>
       <c r="C17" s="8" t="inlineStr">
@@ -861,19 +865,19 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>2026810000020500345</t>
+          <t>2026830000014503061</t>
         </is>
       </c>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>0443063-23.2026.4.05.0000</t>
+          <t>0451459-86.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>20º VF CE</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -883,19 +887,19 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>2026810000020500388</t>
+          <t>2026800000014507369</t>
         </is>
       </c>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>0440332-54.2026.4.05.0000</t>
+          <t>0452226-27.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>33º VF CE</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="C19" s="8" t="inlineStr">
@@ -905,19 +909,19 @@
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>2026810000033500154</t>
+          <t>2026800000014508334</t>
         </is>
       </c>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>0440886-86.2026.4.05.0000</t>
+          <t>0452009-81.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>4º VF SE</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
@@ -927,190 +931,190 @@
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>2026850000004500380</t>
+          <t>2026800000014508108</t>
         </is>
       </c>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>0432087-54.2026.4.05.0000</t>
+          <t>0450523-61.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>33º VF CE</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="C21" s="8" t="inlineStr">
         <is>
-          <t>Caixa Econômica Federal</t>
+          <t>Banco do Brasil S/A</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
         <is>
-          <t>2026810000033500131</t>
+          <t>2026800000014506466</t>
         </is>
       </c>
     </row>
     <row r="22" ht="22" customHeight="1">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>0421015-70.2026.4.05.0000</t>
+          <t>0448852-03.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>9º VF PE</t>
+          <t>20º VF CE</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>Caixa Econômica Federal</t>
+          <t>Banco do Brasil S/A</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>2026840002009501445</t>
+          <t>2026810000020500409</t>
         </is>
       </c>
     </row>
     <row r="23" ht="22" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>0432115-22.2026.4.05.0000</t>
+          <t>0445686-60.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>6º VF AL</t>
+          <t>7º VF RN</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Caixa Econômica Federal</t>
+          <t>Banco do Brasil S/A</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
         <is>
-          <t>2026800000006508048</t>
+          <t>2026840000007506232</t>
         </is>
       </c>
     </row>
     <row r="24" ht="22" customHeight="1">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>0429599-29.2026.4.05.0000</t>
+          <t>0445352-26.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>9º VF AL</t>
+          <t>6º VF AL</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>Caixa Econômica Federal</t>
+          <t>Banco do Brasil S/A</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>2026800000009504071</t>
+          <t>2026800000006508585</t>
         </is>
       </c>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>0429600-14.2026.4.05.0000</t>
+          <t>0447817-08.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>9º VF AL</t>
+          <t>9º VF PB</t>
         </is>
       </c>
       <c r="C25" s="8" t="inlineStr">
         <is>
-          <t>Caixa Econômica Federal</t>
+          <t>Banco do Brasil S/A</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
         <is>
-          <t>2026800000009504072</t>
+          <t>2026820001009502477</t>
         </is>
       </c>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>0432006-08.2026.4.05.0000</t>
+          <t>0448842-56.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>11º VF AL</t>
+          <t>20º VF CE</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>Caixa Econômica Federal</t>
+          <t>Banco do Brasil S/A</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>2026800003011505673</t>
+          <t>2026810000020500407</t>
         </is>
       </c>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>0429605-36.2026.4.05.0000</t>
+          <t>0445358-33.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>9º VF AL</t>
+          <t>6º VF AL</t>
         </is>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
-          <t>Caixa Econômica Federal</t>
+          <t>Banco do Brasil S/A</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
-          <t>2026800000009504043</t>
+          <t>2026800000006508591</t>
         </is>
       </c>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>0433003-88.2026.4.05.0000</t>
+          <t>0445470-02.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>4º VF SE</t>
+          <t>6º VF AL</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>Caixa Econômica Federal</t>
+          <t>Banco do Brasil S/A</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>2026850000004500263</t>
+          <t>2026800000006508699</t>
         </is>
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>0429807-13.2026.4.05.0000</t>
+          <t>0448213-82.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -1120,90 +1124,90 @@
       </c>
       <c r="C29" s="8" t="inlineStr">
         <is>
-          <t>Caixa Econômica Federal</t>
+          <t>Banco do Brasil S/A</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
         <is>
-          <t>2026800000009504294</t>
+          <t>2026800000009503783</t>
         </is>
       </c>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>0421013-03.2026.4.05.0000</t>
+          <t>0445489-08.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>9º VF PE</t>
+          <t>6º VF AL</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>Caixa Econômica Federal</t>
+          <t>Banco do Brasil S/A</t>
         </is>
       </c>
       <c r="D30" s="4" t="inlineStr">
         <is>
-          <t>2026840002009501374</t>
+          <t>2026800000006508650</t>
         </is>
       </c>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>0432271-10.2026.4.05.0000</t>
+          <t>0448848-63.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
         <is>
-          <t>1º VF PB</t>
+          <t>20º VF CE</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Caixa Econômica Federal</t>
+          <t>Banco do Brasil S/A</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>2026820000001500268</t>
+          <t>2026810000020500411</t>
         </is>
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>0435911-21.2026.4.05.0000</t>
+          <t>0445330-65.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B32" s="4" t="inlineStr">
         <is>
-          <t>3º VF PE</t>
+          <t>6º VF AL</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>Caixa Econômica Federal</t>
+          <t>Banco do Brasil S/A</t>
         </is>
       </c>
       <c r="D32" s="4" t="inlineStr">
         <is>
-          <t>2026850000003500131</t>
+          <t>2026800000006508563</t>
         </is>
       </c>
     </row>
     <row r="33" ht="22" customHeight="1">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>0436433-48.2026.4.05.0000</t>
+          <t>0440400-04.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>6º VF AL</t>
+          <t>25º VF PE</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
@@ -1213,19 +1217,19 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>2026800000006508281</t>
+          <t>2026830006025502135</t>
         </is>
       </c>
     </row>
     <row r="34" ht="22" customHeight="1">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>0440400-04.2026.4.05.0000</t>
+          <t>0444257-58.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B34" s="4" t="inlineStr">
         <is>
-          <t>25º VF PE</t>
+          <t>9º VF CE</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -1235,19 +1239,19 @@
       </c>
       <c r="D34" s="4" t="inlineStr">
         <is>
-          <t>2026830006025502135</t>
+          <t>2026810000009500096</t>
         </is>
       </c>
     </row>
     <row r="35" ht="22" customHeight="1">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>0442485-60.2026.4.05.0000</t>
+          <t>0443063-23.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
         <is>
-          <t>14º VF PE</t>
+          <t>20º VF CE</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
@@ -1257,19 +1261,19 @@
       </c>
       <c r="D35" s="7" t="inlineStr">
         <is>
-          <t>2026830000014503418</t>
+          <t>2026810000020500388</t>
         </is>
       </c>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>0445330-65.2026.4.05.0000</t>
+          <t>0442485-60.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B36" s="4" t="inlineStr">
         <is>
-          <t>6º VF AL</t>
+          <t>14º VF PE</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
@@ -1279,19 +1283,19 @@
       </c>
       <c r="D36" s="4" t="inlineStr">
         <is>
-          <t>2026800000006508563</t>
+          <t>2026830000014503418</t>
         </is>
       </c>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>0439583-37.2026.4.05.0000</t>
+          <t>0440202-64.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>12º VF AL</t>
+          <t>19º VF PE</t>
         </is>
       </c>
       <c r="C37" s="8" t="inlineStr">
@@ -1301,19 +1305,19 @@
       </c>
       <c r="D37" s="7" t="inlineStr">
         <is>
-          <t>2026800001012503362</t>
+          <t>2026830000019502593</t>
         </is>
       </c>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>0439844-02.2026.4.05.0000</t>
+          <t>0443066-75.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B38" s="4" t="inlineStr">
         <is>
-          <t>6º VF AL</t>
+          <t>20º VF CE</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
@@ -1323,19 +1327,19 @@
       </c>
       <c r="D38" s="4" t="inlineStr">
         <is>
-          <t>2026800000006508482</t>
+          <t>2026810000020500391</t>
         </is>
       </c>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>0436398-88.2026.4.05.0000</t>
+          <t>0440333-39.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>6º VF AL</t>
+          <t>33º VF CE</t>
         </is>
       </c>
       <c r="C39" s="8" t="inlineStr">
@@ -1345,19 +1349,19 @@
       </c>
       <c r="D39" s="7" t="inlineStr">
         <is>
-          <t>2026800000006508316</t>
+          <t>2026810000033500155</t>
         </is>
       </c>
     </row>
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>0444257-58.2026.4.05.0000</t>
+          <t>0440332-54.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B40" s="4" t="inlineStr">
         <is>
-          <t>9º VF CE</t>
+          <t>33º VF CE</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
@@ -1367,19 +1371,19 @@
       </c>
       <c r="D40" s="4" t="inlineStr">
         <is>
-          <t>2026810000009500096</t>
+          <t>2026810000033500154</t>
         </is>
       </c>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>0440202-64.2026.4.05.0000</t>
+          <t>0440886-86.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>19º VF PE</t>
+          <t>4º VF SE</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
@@ -1389,19 +1393,19 @@
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>2026830000019502593</t>
+          <t>2026850000004500380</t>
         </is>
       </c>
     </row>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>0445352-26.2026.4.05.0000</t>
+          <t>0440075-29.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B42" s="4" t="inlineStr">
         <is>
-          <t>6º VF AL</t>
+          <t>20º VF CE</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
@@ -1411,63 +1415,63 @@
       </c>
       <c r="D42" s="4" t="inlineStr">
         <is>
-          <t>2026800000006508585</t>
+          <t>2026810000020500345</t>
         </is>
       </c>
     </row>
     <row r="43" ht="22" customHeight="1">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>0445358-33.2026.4.05.0000</t>
+          <t>0435911-21.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>6º VF AL</t>
+          <t>3º VF PE</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>2026800000006508591</t>
+          <t>2026850000003500131</t>
         </is>
       </c>
     </row>
     <row r="44" ht="22" customHeight="1">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>0445489-08.2026.4.05.0000</t>
+          <t>0433003-88.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B44" s="4" t="inlineStr">
         <is>
-          <t>6º VF AL</t>
+          <t>4º VF SE</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D44" s="4" t="inlineStr">
         <is>
-          <t>2026800000006508650</t>
+          <t>2026850000004500263</t>
         </is>
       </c>
     </row>
     <row r="45" ht="22" customHeight="1">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>0451653-86.2026.4.05.0000</t>
+          <t>0436433-48.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>6º VF AL</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
@@ -1477,19 +1481,19 @@
       </c>
       <c r="D45" s="7" t="inlineStr">
         <is>
-          <t>2026800000014507587</t>
+          <t>2026800000006508281</t>
         </is>
       </c>
     </row>
     <row r="46" ht="22" customHeight="1">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>0447817-08.2026.4.05.0000</t>
+          <t>0439583-37.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B46" s="4" t="inlineStr">
         <is>
-          <t>9º VF PB</t>
+          <t>12º VF AL</t>
         </is>
       </c>
       <c r="C46" s="5" t="inlineStr">
@@ -1499,14 +1503,14 @@
       </c>
       <c r="D46" s="4" t="inlineStr">
         <is>
-          <t>2026820001009502477</t>
+          <t>2026800001012503362</t>
         </is>
       </c>
     </row>
     <row r="47" ht="22" customHeight="1">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>0445470-02.2026.4.05.0000</t>
+          <t>0439844-02.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -1521,19 +1525,19 @@
       </c>
       <c r="D47" s="7" t="inlineStr">
         <is>
-          <t>2026800000006508699</t>
+          <t>2026800000006508482</t>
         </is>
       </c>
     </row>
     <row r="48" ht="22" customHeight="1">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>0451459-86.2026.4.05.0000</t>
+          <t>0436398-88.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B48" s="4" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>6º VF AL</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
@@ -1543,327 +1547,327 @@
       </c>
       <c r="D48" s="4" t="inlineStr">
         <is>
-          <t>2026800000014507369</t>
+          <t>2026800000006508316</t>
         </is>
       </c>
     </row>
     <row r="49" ht="22" customHeight="1">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>0450523-61.2026.4.05.0000</t>
+          <t>0433722-70.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>20º VF CE</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>2026800000014506466</t>
+          <t>2026810000020500262</t>
         </is>
       </c>
     </row>
     <row r="50" ht="22" customHeight="1">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>0450167-66.2026.4.05.0000</t>
+          <t>0434796-62.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B50" s="4" t="inlineStr">
         <is>
-          <t>14º VF PE</t>
+          <t>33º VF CE</t>
         </is>
       </c>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D50" s="4" t="inlineStr">
         <is>
-          <t>2026830000014503061</t>
+          <t>2026810000033500132</t>
         </is>
       </c>
     </row>
     <row r="51" ht="22" customHeight="1">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>0448213-82.2026.4.05.0000</t>
+          <t>0432271-10.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>9º VF AL</t>
+          <t>1º VF PB</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>2026800000009503783</t>
+          <t>2026820000001500268</t>
         </is>
       </c>
     </row>
     <row r="52" ht="22" customHeight="1">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>0451747-34.2026.4.05.0000</t>
+          <t>0432115-22.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B52" s="4" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>6º VF AL</t>
         </is>
       </c>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D52" s="4" t="inlineStr">
         <is>
-          <t>2026800000014507488</t>
+          <t>2026800000006508048</t>
         </is>
       </c>
     </row>
     <row r="53" ht="22" customHeight="1">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>0452536-33.2026.4.05.0000</t>
+          <t>0432087-54.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>33º VF CE</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>2026800000014508690</t>
+          <t>2026810000033500131</t>
         </is>
       </c>
     </row>
     <row r="54" ht="22" customHeight="1">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>0452009-81.2026.4.05.0000</t>
+          <t>0429807-13.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B54" s="4" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>9º VF AL</t>
         </is>
       </c>
       <c r="C54" s="5" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D54" s="4" t="inlineStr">
         <is>
-          <t>2026800000014508108</t>
+          <t>2026800000009504294</t>
         </is>
       </c>
     </row>
     <row r="55" ht="22" customHeight="1">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>0452256-62.2026.4.05.0000</t>
+          <t>0429596-74.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>9º VF AL</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
         <is>
-          <t>2026800000014506443</t>
+          <t>2026800000009504063</t>
         </is>
       </c>
     </row>
     <row r="56" ht="22" customHeight="1">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>0452601-28.2026.4.05.0000</t>
+          <t>0429598-44.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B56" s="4" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>9º VF AL</t>
         </is>
       </c>
       <c r="C56" s="5" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D56" s="4" t="inlineStr">
         <is>
-          <t>2026800000014508618</t>
+          <t>2026800000009504069</t>
         </is>
       </c>
     </row>
     <row r="57" ht="22" customHeight="1">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>0452854-16.2026.4.05.0000</t>
+          <t>0429605-36.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>9º VF AL</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
         <is>
-          <t>2026800000014508192</t>
+          <t>2026800000009504043</t>
         </is>
       </c>
     </row>
     <row r="58" ht="22" customHeight="1">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>0452384-82.2026.4.05.0000</t>
+          <t>0432006-08.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B58" s="4" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>11º VF AL</t>
         </is>
       </c>
       <c r="C58" s="5" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D58" s="4" t="inlineStr">
         <is>
-          <t>2026800000014507635</t>
+          <t>2026800003011505673</t>
         </is>
       </c>
     </row>
     <row r="59" ht="22" customHeight="1">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>0452501-73.2026.4.05.0000</t>
+          <t>0429395-82.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>9º VF AL</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
         <is>
-          <t>2026800000014508173</t>
+          <t>2026800000009503544</t>
         </is>
       </c>
     </row>
     <row r="60" ht="22" customHeight="1">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>0452306-88.2026.4.05.0000</t>
+          <t>0429599-29.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B60" s="4" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>9º VF AL</t>
         </is>
       </c>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D60" s="4" t="inlineStr">
         <is>
-          <t>2026800000014508366</t>
+          <t>2026800000009504071</t>
         </is>
       </c>
     </row>
     <row r="61" ht="22" customHeight="1">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>0452735-55.2026.4.05.0000</t>
+          <t>0429600-14.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>9º VF AL</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
         <is>
-          <t>2026800000014508926</t>
+          <t>2026800000009504072</t>
         </is>
       </c>
     </row>
     <row r="62" ht="22" customHeight="1">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>0454207-91.2026.4.05.0000</t>
+          <t>0429381-98.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B62" s="4" t="inlineStr">
         <is>
-          <t>7º VF RN</t>
+          <t>9º VF AL</t>
         </is>
       </c>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D62" s="4" t="inlineStr">
         <is>
-          <t>2026840000007505433</t>
+          <t>2026800000009503562</t>
         </is>
       </c>
     </row>
     <row r="63" ht="22" customHeight="1">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>0422323-44.2026.4.05.0000</t>
+          <t>0429144-64.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>7º VF RN</t>
+          <t>9º VF AL</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
@@ -1873,41 +1877,41 @@
       </c>
       <c r="D63" s="7" t="inlineStr">
         <is>
-          <t>2026840000007503056</t>
+          <t>2026800000009503319</t>
         </is>
       </c>
     </row>
     <row r="64" ht="22" customHeight="1">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>0459281-29.2026.4.05.0000</t>
+          <t>0429031-13.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B64" s="4" t="inlineStr">
         <is>
-          <t>14º VF PE</t>
+          <t>9º VF AL</t>
         </is>
       </c>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D64" s="4" t="inlineStr">
         <is>
-          <t>2026830000014504238</t>
+          <t>2026800000009502988</t>
         </is>
       </c>
     </row>
     <row r="65" ht="22" customHeight="1">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>0426515-20.2026.4.05.0000</t>
+          <t>0429143-79.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>6º VF AL</t>
+          <t>9º VF AL</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
@@ -1917,63 +1921,63 @@
       </c>
       <c r="D65" s="7" t="inlineStr">
         <is>
-          <t>2026800000006507810</t>
+          <t>2026800000009503318</t>
         </is>
       </c>
     </row>
     <row r="66" ht="22" customHeight="1">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>0459836-46.2026.4.05.0000</t>
+          <t>0428095-85.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B66" s="4" t="inlineStr">
         <is>
-          <t>3º VF RN</t>
+          <t>10º VF AL</t>
         </is>
       </c>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D66" s="4" t="inlineStr">
         <is>
-          <t>2026840000003503607</t>
+          <t>2026800001010503452</t>
         </is>
       </c>
     </row>
     <row r="67" ht="22" customHeight="1">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>0461413-59.2026.4.05.0000</t>
+          <t>0428241-29.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>34º VF PE</t>
+          <t>13º VF AL</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
         <is>
-          <t>2026830012034500718</t>
+          <t>2026800000013500090</t>
         </is>
       </c>
     </row>
     <row r="68" ht="22" customHeight="1">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>0423263-09.2026.4.05.0000</t>
+          <t>0429070-10.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B68" s="4" t="inlineStr">
         <is>
-          <t>7º VF RN</t>
+          <t>9º VF AL</t>
         </is>
       </c>
       <c r="C68" s="5" t="inlineStr">
@@ -1983,63 +1987,63 @@
       </c>
       <c r="D68" s="4" t="inlineStr">
         <is>
-          <t>2026840000007505332</t>
+          <t>2026800000009503137</t>
         </is>
       </c>
     </row>
     <row r="69" ht="22" customHeight="1">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>0458573-76.2026.4.05.0000</t>
+          <t>0427483-50.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>13º VF PE</t>
+          <t>30º VF PE</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
         <is>
-          <t>2026820000013510143</t>
+          <t>2026830011030502090</t>
         </is>
       </c>
     </row>
     <row r="70" ht="22" customHeight="1">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>0458903-73.2026.4.05.0000</t>
+          <t>0426978-59.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B70" s="4" t="inlineStr">
         <is>
-          <t>3º VF PE</t>
+          <t>11º VF AL</t>
         </is>
       </c>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Banco do Brasil S/A</t>
+          <t>Caixa Econômica Federal</t>
         </is>
       </c>
       <c r="D70" s="4" t="inlineStr">
         <is>
-          <t>2026820000003500707</t>
+          <t>2026800003011505648</t>
         </is>
       </c>
     </row>
     <row r="71" ht="22" customHeight="1">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>0422322-59.2026.4.05.0000</t>
+          <t>0426615-72.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>7º VF RN</t>
+          <t>6º VF AL</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
@@ -2049,14 +2053,14 @@
       </c>
       <c r="D71" s="7" t="inlineStr">
         <is>
-          <t>2026840000007503047</t>
+          <t>2026800000006507954</t>
         </is>
       </c>
     </row>
     <row r="72" ht="22" customHeight="1">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>0426615-72.2026.4.05.0000</t>
+          <t>0426618-27.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B72" s="4" t="inlineStr">
@@ -2071,19 +2075,19 @@
       </c>
       <c r="D72" s="4" t="inlineStr">
         <is>
-          <t>2026800000006507954</t>
+          <t>2026800000006507957</t>
         </is>
       </c>
     </row>
     <row r="73" ht="22" customHeight="1">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>0429144-64.2026.4.05.0000</t>
+          <t>0421013-03.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>9º VF AL</t>
+          <t>9º VF PE</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
@@ -2093,19 +2097,19 @@
       </c>
       <c r="D73" s="7" t="inlineStr">
         <is>
-          <t>2026800000009503319</t>
+          <t>2026840002009501374</t>
         </is>
       </c>
     </row>
     <row r="74" ht="22" customHeight="1">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>0426618-27.2026.4.05.0000</t>
+          <t>0423263-09.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B74" s="4" t="inlineStr">
         <is>
-          <t>6º VF AL</t>
+          <t>7º VF RN</t>
         </is>
       </c>
       <c r="C74" s="5" t="inlineStr">
@@ -2115,63 +2119,55 @@
       </c>
       <c r="D74" s="4" t="inlineStr">
         <is>
-          <t>2026800000006507957</t>
+          <t>2026840000007505332</t>
         </is>
       </c>
     </row>
     <row r="75" ht="22" customHeight="1">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>0429070-10.2026.4.05.0000</t>
+          <t>0475186-74.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>9º VF AL</t>
-        </is>
-      </c>
-      <c r="C75" s="8" t="inlineStr">
-        <is>
-          <t>Caixa Econômica Federal</t>
-        </is>
-      </c>
+          <t>2º VF PE</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr"/>
       <c r="D75" s="7" t="inlineStr">
         <is>
-          <t>2026800000009503137</t>
+          <t>2026830000002500313</t>
         </is>
       </c>
     </row>
     <row r="76" ht="22" customHeight="1">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>0428095-85.2026.4.05.0000</t>
+          <t>0473876-33.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B76" s="4" t="inlineStr">
         <is>
-          <t>10º VF AL</t>
-        </is>
-      </c>
-      <c r="C76" s="5" t="inlineStr">
-        <is>
-          <t>Caixa Econômica Federal</t>
-        </is>
-      </c>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C76" s="5" t="inlineStr"/>
       <c r="D76" s="4" t="inlineStr">
         <is>
-          <t>2026800001010503452</t>
+          <t>2026800000009506036</t>
         </is>
       </c>
     </row>
     <row r="77" ht="22" customHeight="1">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>0426978-59.2026.4.05.0000</t>
+          <t>0422323-44.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>11º VF AL</t>
+          <t>7º VF RN</t>
         </is>
       </c>
       <c r="C77" s="8" t="inlineStr">
@@ -2181,19 +2177,19 @@
       </c>
       <c r="D77" s="7" t="inlineStr">
         <is>
-          <t>2026800003011505648</t>
+          <t>2026840000007503056</t>
         </is>
       </c>
     </row>
     <row r="78" ht="22" customHeight="1">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>0427483-50.2026.4.05.0000</t>
+          <t>0422322-59.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B78" s="4" t="inlineStr">
         <is>
-          <t>30º VF PE</t>
+          <t>7º VF RN</t>
         </is>
       </c>
       <c r="C78" s="5" t="inlineStr">
@@ -2203,19 +2199,19 @@
       </c>
       <c r="D78" s="4" t="inlineStr">
         <is>
-          <t>2026830011030502090</t>
+          <t>2026840000007503047</t>
         </is>
       </c>
     </row>
     <row r="79" ht="22" customHeight="1">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>0429143-79.2026.4.05.0000</t>
+          <t>0426515-20.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>9º VF AL</t>
+          <t>6º VF AL</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
@@ -2225,19 +2221,19 @@
       </c>
       <c r="D79" s="7" t="inlineStr">
         <is>
-          <t>2026800000009503318</t>
+          <t>2026800000006507810</t>
         </is>
       </c>
     </row>
     <row r="80" ht="22" customHeight="1">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>0429031-13.2026.4.05.0000</t>
+          <t>0421015-70.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B80" s="4" t="inlineStr">
         <is>
-          <t>9º VF AL</t>
+          <t>9º VF PE</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
@@ -2247,19 +2243,19 @@
       </c>
       <c r="D80" s="4" t="inlineStr">
         <is>
-          <t>2026800000009502988</t>
+          <t>2026840002009501445</t>
         </is>
       </c>
     </row>
     <row r="81" ht="22" customHeight="1">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>0428241-29.2026.4.05.0000</t>
+          <t>0422526-06.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>13º VF AL</t>
+          <t>7º VF RN</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
@@ -2269,14 +2265,14 @@
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>2026800000013500090</t>
+          <t>2026840000007504848</t>
         </is>
       </c>
     </row>
     <row r="82" ht="22" customHeight="1">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>0429381-98.2026.4.05.0000</t>
+          <t>0473889-32.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B82" s="4" t="inlineStr">
@@ -2284,21 +2280,17 @@
           <t>9º VF AL</t>
         </is>
       </c>
-      <c r="C82" s="5" t="inlineStr">
-        <is>
-          <t>Caixa Econômica Federal</t>
-        </is>
-      </c>
+      <c r="C82" s="5" t="inlineStr"/>
       <c r="D82" s="4" t="inlineStr">
         <is>
-          <t>2026800000009503562</t>
+          <t>2026800000009506209</t>
         </is>
       </c>
     </row>
     <row r="83" ht="22" customHeight="1">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>0429395-82.2026.4.05.0000</t>
+          <t>0473849-50.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
@@ -2306,286 +2298,262 @@
           <t>9º VF AL</t>
         </is>
       </c>
-      <c r="C83" s="8" t="inlineStr">
-        <is>
-          <t>Caixa Econômica Federal</t>
-        </is>
-      </c>
+      <c r="C83" s="8" t="inlineStr"/>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>2026800000009503544</t>
+          <t>2026800000009505857</t>
         </is>
       </c>
     </row>
     <row r="84" ht="22" customHeight="1">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>0464899-52.2026.4.05.0000</t>
+          <t>0472989-49.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B84" s="4" t="inlineStr">
         <is>
-          <t>14º VF PE</t>
+          <t>14º VF CE</t>
         </is>
       </c>
       <c r="C84" s="5" t="inlineStr"/>
       <c r="D84" s="4" t="inlineStr">
         <is>
-          <t>2026830000014504627</t>
+          <t>2026810000014503814</t>
         </is>
       </c>
     </row>
     <row r="85" ht="22" customHeight="1">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>0466785-86.2026.4.05.0000</t>
+          <t>0471731-04.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>7º VF AL</t>
+          <t>9º VF AL</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr"/>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>2026800002007503620</t>
+          <t>2026800000009505547</t>
         </is>
       </c>
     </row>
     <row r="86" ht="22" customHeight="1">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>0429598-44.2026.4.05.0000</t>
+          <t>0470950-79.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B86" s="4" t="inlineStr">
         <is>
-          <t>9º VF AL</t>
-        </is>
-      </c>
-      <c r="C86" s="5" t="inlineStr">
-        <is>
-          <t>Caixa Econômica Federal</t>
-        </is>
-      </c>
+          <t>27º VF PE</t>
+        </is>
+      </c>
+      <c r="C86" s="5" t="inlineStr"/>
       <c r="D86" s="4" t="inlineStr">
         <is>
-          <t>2026800000009504069</t>
+          <t>2026830009027502123</t>
         </is>
       </c>
     </row>
     <row r="87" ht="22" customHeight="1">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>0464849-26.2026.4.05.0000</t>
+          <t>0472988-64.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>7º VF RN</t>
+          <t>14º VF CE</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr"/>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>2026840000007505544</t>
+          <t>2026810000014503813</t>
         </is>
       </c>
     </row>
     <row r="88" ht="22" customHeight="1">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>0464331-36.2026.4.05.0000</t>
+          <t>0471777-90.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B88" s="4" t="inlineStr">
         <is>
-          <t>6º VF AL</t>
+          <t>9º VF AL</t>
         </is>
       </c>
       <c r="C88" s="5" t="inlineStr"/>
       <c r="D88" s="4" t="inlineStr">
         <is>
-          <t>2026800000006509055</t>
+          <t>2026800000009505562</t>
         </is>
       </c>
     </row>
     <row r="89" ht="22" customHeight="1">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>0464605-97.2026.4.05.0000</t>
+          <t>0471775-23.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
         <is>
-          <t>6º VF AL</t>
+          <t>9º VF AL</t>
         </is>
       </c>
       <c r="C89" s="8" t="inlineStr"/>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>2026800000006509381</t>
+          <t>2026800000009505560</t>
         </is>
       </c>
     </row>
     <row r="90" ht="22" customHeight="1">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>0429596-74.2026.4.05.0000</t>
+          <t>0466785-86.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B90" s="4" t="inlineStr">
         <is>
-          <t>9º VF AL</t>
-        </is>
-      </c>
-      <c r="C90" s="5" t="inlineStr">
-        <is>
-          <t>Caixa Econômica Federal</t>
-        </is>
-      </c>
+          <t>7º VF AL</t>
+        </is>
+      </c>
+      <c r="C90" s="5" t="inlineStr"/>
       <c r="D90" s="4" t="inlineStr">
         <is>
-          <t>2026800000009504063</t>
+          <t>2026800002007503620</t>
         </is>
       </c>
     </row>
     <row r="91" ht="22" customHeight="1">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>0464356-49.2026.4.05.0000</t>
+          <t>0468287-60.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>6º VF AL</t>
+          <t>16º VF PE</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr"/>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>2026800000006509082</t>
+          <t>2026830002016500799</t>
         </is>
       </c>
     </row>
     <row r="92" ht="22" customHeight="1">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>0464329-66.2026.4.05.0000</t>
+          <t>0464899-52.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B92" s="4" t="inlineStr">
         <is>
-          <t>6º VF AL</t>
+          <t>14º VF PE</t>
         </is>
       </c>
       <c r="C92" s="5" t="inlineStr"/>
       <c r="D92" s="4" t="inlineStr">
         <is>
-          <t>2026800000006509053</t>
+          <t>2026830000014504627</t>
         </is>
       </c>
     </row>
     <row r="93" ht="22" customHeight="1">
       <c r="A93" s="6" t="inlineStr">
         <is>
-          <t>0461673-39.2026.4.05.0000</t>
+          <t>0464356-49.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>30º VF PE</t>
+          <t>6º VF AL</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr"/>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>2026830011030502351</t>
+          <t>2026800000006509082</t>
         </is>
       </c>
     </row>
     <row r="94" ht="22" customHeight="1">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>0418861-79.2026.4.05.0000</t>
+          <t>0464849-26.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B94" s="4" t="inlineStr">
         <is>
-          <t>10º VF AL</t>
-        </is>
-      </c>
-      <c r="C94" s="5" t="inlineStr">
-        <is>
-          <t>Banco do Brasil S/A</t>
-        </is>
-      </c>
+          <t>7º VF RN</t>
+        </is>
+      </c>
+      <c r="C94" s="5" t="inlineStr"/>
       <c r="D94" s="4" t="inlineStr">
         <is>
-          <t>2026800001010502803</t>
+          <t>2026840000007505544</t>
         </is>
       </c>
     </row>
     <row r="95" ht="22" customHeight="1">
       <c r="A95" s="6" t="inlineStr">
         <is>
-          <t>0419484-46.2026.4.05.0000</t>
+          <t>0464605-97.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>10º VF AL</t>
-        </is>
-      </c>
-      <c r="C95" s="8" t="inlineStr">
-        <is>
-          <t>Banco do Brasil S/A</t>
-        </is>
-      </c>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C95" s="8" t="inlineStr"/>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>2026800001010503210</t>
+          <t>2026800000006509381</t>
         </is>
       </c>
     </row>
     <row r="96" ht="22" customHeight="1">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>0461780-83.2026.4.05.0000</t>
+          <t>0464329-66.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B96" s="4" t="inlineStr">
         <is>
-          <t>9º VF AL</t>
+          <t>6º VF AL</t>
         </is>
       </c>
       <c r="C96" s="5" t="inlineStr"/>
       <c r="D96" s="4" t="inlineStr">
         <is>
-          <t>2026800000009504875</t>
+          <t>2026800000006509053</t>
         </is>
       </c>
     </row>
     <row r="97" ht="22" customHeight="1">
       <c r="A97" s="6" t="inlineStr">
         <is>
-          <t>0401993-26.2026.4.05.0000</t>
+          <t>0461780-83.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B97" s="7" t="inlineStr">
         <is>
-          <t>2º VF PE</t>
-        </is>
-      </c>
-      <c r="C97" s="8" t="inlineStr">
-        <is>
-          <t>Caixa Econômica Federal</t>
-        </is>
-      </c>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C97" s="8" t="inlineStr"/>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>2026830000002500220</t>
+          <t>2026800000009504875</t>
         </is>
       </c>
     </row>
@@ -2610,66 +2578,2258 @@
     <row r="99" ht="22" customHeight="1">
       <c r="A99" s="6" t="inlineStr">
         <is>
-          <t>0411960-95.2026.4.05.0000</t>
+          <t>0461673-39.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
-          <t>20º VF CE</t>
-        </is>
-      </c>
-      <c r="C99" s="8" t="inlineStr">
-        <is>
-          <t>Banco do Brasil S/A</t>
-        </is>
-      </c>
+          <t>30º VF PE</t>
+        </is>
+      </c>
+      <c r="C99" s="8" t="inlineStr"/>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>2026810000020500292</t>
+          <t>2026830011030502351</t>
         </is>
       </c>
     </row>
     <row r="100" ht="22" customHeight="1">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>0393292-76.2026.4.05.0000</t>
+          <t>0464331-36.2026.4.05.0000</t>
         </is>
       </c>
       <c r="B100" s="4" t="inlineStr">
         <is>
-          <t>2º VF SE</t>
-        </is>
-      </c>
-      <c r="C100" s="5" t="inlineStr">
-        <is>
-          <t>Caixa Econômica Federal</t>
-        </is>
-      </c>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C100" s="5" t="inlineStr"/>
       <c r="D100" s="4" t="inlineStr">
         <is>
-          <t>2026850000002500075</t>
+          <t>2026800000006509055</t>
         </is>
       </c>
     </row>
     <row r="101" ht="22" customHeight="1">
       <c r="A101" s="6" t="inlineStr">
         <is>
+          <t>0401993-26.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B101" s="7" t="inlineStr">
+        <is>
+          <t>2º VF PE</t>
+        </is>
+      </c>
+      <c r="C101" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D101" s="7" t="inlineStr">
+        <is>
+          <t>2026830000002500220</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="22" customHeight="1">
+      <c r="A102" s="3" t="inlineStr">
+        <is>
+          <t>0393292-76.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B102" s="4" t="inlineStr">
+        <is>
+          <t>2º VF SE</t>
+        </is>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>2026850000002500075</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="22" customHeight="1">
+      <c r="A103" s="6" t="inlineStr">
+        <is>
+          <t>0397418-72.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B103" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C103" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D103" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006506745</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="22" customHeight="1">
+      <c r="A104" s="3" t="inlineStr">
+        <is>
+          <t>0418861-79.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B104" s="4" t="inlineStr">
+        <is>
+          <t>10º VF AL</t>
+        </is>
+      </c>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>2026800001010502803</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="22" customHeight="1">
+      <c r="A105" s="6" t="inlineStr">
+        <is>
+          <t>0419484-46.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B105" s="7" t="inlineStr">
+        <is>
+          <t>10º VF AL</t>
+        </is>
+      </c>
+      <c r="C105" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D105" s="7" t="inlineStr">
+        <is>
+          <t>2026800001010503210</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="22" customHeight="1">
+      <c r="A106" s="3" t="inlineStr">
+        <is>
           <t>0397570-23.2026.4.05.0000</t>
         </is>
       </c>
-      <c r="B101" s="7" t="inlineStr">
+      <c r="B106" s="4" t="inlineStr">
         <is>
           <t>4º VF SE</t>
         </is>
       </c>
-      <c r="C101" s="8" t="inlineStr">
-        <is>
-          <t>Banco do Brasil S/A</t>
-        </is>
-      </c>
-      <c r="D101" s="7" t="inlineStr">
+      <c r="C106" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
         <is>
           <t>2026850000004500323</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="22" customHeight="1">
+      <c r="A107" s="6" t="inlineStr">
+        <is>
+          <t>0395901-32.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B107" s="7" t="inlineStr">
+        <is>
+          <t>8º VF SE</t>
+        </is>
+      </c>
+      <c r="C107" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D107" s="7" t="inlineStr">
+        <is>
+          <t>2026850003008500879</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="22" customHeight="1">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>0419505-22.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B108" s="4" t="inlineStr">
+        <is>
+          <t>10º VF AL</t>
+        </is>
+      </c>
+      <c r="C108" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>2026800001010503117</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="22" customHeight="1">
+      <c r="A109" s="6" t="inlineStr">
+        <is>
+          <t>0397416-05.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B109" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C109" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D109" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006506743</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="22" customHeight="1">
+      <c r="A110" s="3" t="inlineStr">
+        <is>
+          <t>0398704-85.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>4º VF SE</t>
+        </is>
+      </c>
+      <c r="C110" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>2026850000004500325</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="22" customHeight="1">
+      <c r="A111" s="6" t="inlineStr">
+        <is>
+          <t>0411960-95.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B111" s="7" t="inlineStr">
+        <is>
+          <t>20º VF CE</t>
+        </is>
+      </c>
+      <c r="C111" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D111" s="7" t="inlineStr">
+        <is>
+          <t>2026810000020500292</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="22" customHeight="1">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>0411692-41.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B112" s="4" t="inlineStr">
+        <is>
+          <t>10º VF AL</t>
+        </is>
+      </c>
+      <c r="C112" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>2026800001010502610</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="22" customHeight="1">
+      <c r="A113" s="6" t="inlineStr">
+        <is>
+          <t>0416419-43.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B113" s="7" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C113" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D113" s="7" t="inlineStr">
+        <is>
+          <t>2026800000014505678</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="22" customHeight="1">
+      <c r="A114" s="3" t="inlineStr">
+        <is>
+          <t>0385881-79.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B114" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006506438</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="22" customHeight="1">
+      <c r="A115" s="6" t="inlineStr">
+        <is>
+          <t>0385879-12.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B115" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C115" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D115" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006506436</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="22" customHeight="1">
+      <c r="A116" s="3" t="inlineStr">
+        <is>
+          <t>0398845-07.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B116" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C116" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006506880</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="22" customHeight="1">
+      <c r="A117" s="6" t="inlineStr">
+        <is>
+          <t>0396665-18.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B117" s="7" t="inlineStr">
+        <is>
+          <t>4º VF SE</t>
+        </is>
+      </c>
+      <c r="C117" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D117" s="7" t="inlineStr">
+        <is>
+          <t>2026850000004500310</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="22" customHeight="1">
+      <c r="A118" s="3" t="inlineStr">
+        <is>
+          <t>0397173-61.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B118" s="4" t="inlineStr">
+        <is>
+          <t>29º VF CE</t>
+        </is>
+      </c>
+      <c r="C118" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>2026810001029503519</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="22" customHeight="1">
+      <c r="A119" s="6" t="inlineStr">
+        <is>
+          <t>0385165-52.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B119" s="7" t="inlineStr">
+        <is>
+          <t>20º VF CE</t>
+        </is>
+      </c>
+      <c r="C119" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D119" s="7" t="inlineStr">
+        <is>
+          <t>2026810000020500234</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="22" customHeight="1">
+      <c r="A120" s="3" t="inlineStr">
+        <is>
+          <t>0413774-45.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B120" s="4" t="inlineStr">
+        <is>
+          <t>15º VF PE</t>
+        </is>
+      </c>
+      <c r="C120" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="inlineStr">
+        <is>
+          <t>2026830000015504639</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="22" customHeight="1">
+      <c r="A121" s="6" t="inlineStr">
+        <is>
+          <t>0395388-64.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B121" s="7" t="inlineStr">
+        <is>
+          <t>8º VF PE</t>
+        </is>
+      </c>
+      <c r="C121" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D121" s="7" t="inlineStr">
+        <is>
+          <t>2026830008008503840</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="22" customHeight="1">
+      <c r="A122" s="3" t="inlineStr">
+        <is>
+          <t>0395171-21.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>20º VF CE</t>
+        </is>
+      </c>
+      <c r="C122" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>2026810000020500248</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="22" customHeight="1">
+      <c r="A123" s="6" t="inlineStr">
+        <is>
+          <t>0418215-69.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B123" s="7" t="inlineStr">
+        <is>
+          <t>3º VF PE</t>
+        </is>
+      </c>
+      <c r="C123" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D123" s="7" t="inlineStr">
+        <is>
+          <t>2026850000003500142</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="22" customHeight="1">
+      <c r="A124" s="3" t="inlineStr">
+        <is>
+          <t>0418214-84.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B124" s="4" t="inlineStr">
+        <is>
+          <t>3º VF PE</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>2026850000003500141</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="22" customHeight="1">
+      <c r="A125" s="6" t="inlineStr">
+        <is>
+          <t>0416217-66.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B125" s="7" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C125" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D125" s="7" t="inlineStr">
+        <is>
+          <t>2026800000014506904</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="22" customHeight="1">
+      <c r="A126" s="3" t="inlineStr">
+        <is>
+          <t>0418213-02.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B126" s="4" t="inlineStr">
+        <is>
+          <t>3º VF PE</t>
+        </is>
+      </c>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D126" s="4" t="inlineStr">
+        <is>
+          <t>2026850000003500140</t>
+        </is>
+      </c>
+    </row>
+    <row r="127" ht="22" customHeight="1">
+      <c r="A127" s="6" t="inlineStr">
+        <is>
+          <t>0415408-76.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B127" s="7" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C127" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D127" s="7" t="inlineStr">
+        <is>
+          <t>2026800000014505481</t>
+        </is>
+      </c>
+    </row>
+    <row r="128" ht="22" customHeight="1">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
+          <t>0415938-80.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B128" s="4" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C128" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>2026800000014506144</t>
+        </is>
+      </c>
+    </row>
+    <row r="129" ht="22" customHeight="1">
+      <c r="A129" s="6" t="inlineStr">
+        <is>
+          <t>0416167-40.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B129" s="7" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C129" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D129" s="7" t="inlineStr">
+        <is>
+          <t>2026800000014506830</t>
+        </is>
+      </c>
+    </row>
+    <row r="130" ht="22" customHeight="1">
+      <c r="A130" s="3" t="inlineStr">
+        <is>
+          <t>0416403-89.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B130" s="4" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C130" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D130" s="4" t="inlineStr">
+        <is>
+          <t>2026800000014505576</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="22" customHeight="1">
+      <c r="A131" s="6" t="inlineStr">
+        <is>
+          <t>0416377-91.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B131" s="7" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C131" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D131" s="7" t="inlineStr">
+        <is>
+          <t>2026800000014507133</t>
+        </is>
+      </c>
+    </row>
+    <row r="132" ht="22" customHeight="1">
+      <c r="A132" s="3" t="inlineStr">
+        <is>
+          <t>0416318-06.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B132" s="4" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C132" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D132" s="4" t="inlineStr">
+        <is>
+          <t>2026800000014505802</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="22" customHeight="1">
+      <c r="A133" s="6" t="inlineStr">
+        <is>
+          <t>0410094-52.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B133" s="7" t="inlineStr">
+        <is>
+          <t>32º VF PE</t>
+        </is>
+      </c>
+      <c r="C133" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D133" s="7" t="inlineStr">
+        <is>
+          <t>2026830005032502386</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="22" customHeight="1">
+      <c r="A134" s="3" t="inlineStr">
+        <is>
+          <t>0415623-52.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B134" s="4" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C134" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D134" s="4" t="inlineStr">
+        <is>
+          <t>2026800000014505747</t>
+        </is>
+      </c>
+    </row>
+    <row r="135" ht="22" customHeight="1">
+      <c r="A135" s="6" t="inlineStr">
+        <is>
+          <t>0384043-04.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B135" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C135" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D135" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006506233</t>
+        </is>
+      </c>
+    </row>
+    <row r="136" ht="22" customHeight="1">
+      <c r="A136" s="3" t="inlineStr">
+        <is>
+          <t>0384023-13.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B136" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C136" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D136" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006506261</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="22" customHeight="1">
+      <c r="A137" s="6" t="inlineStr">
+        <is>
+          <t>0383992-90.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B137" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C137" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D137" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006506204</t>
+        </is>
+      </c>
+    </row>
+    <row r="138" ht="22" customHeight="1">
+      <c r="A138" s="3" t="inlineStr">
+        <is>
+          <t>0416599-59.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C138" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D138" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006507490</t>
+        </is>
+      </c>
+    </row>
+    <row r="139" ht="22" customHeight="1">
+      <c r="A139" s="6" t="inlineStr">
+        <is>
+          <t>0415009-47.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B139" s="7" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C139" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D139" s="7" t="inlineStr">
+        <is>
+          <t>2026800000014504674</t>
+        </is>
+      </c>
+    </row>
+    <row r="140" ht="22" customHeight="1">
+      <c r="A140" s="3" t="inlineStr">
+        <is>
+          <t>0395679-64.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t>7º VF PE</t>
+        </is>
+      </c>
+      <c r="C140" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D140" s="4" t="inlineStr">
+        <is>
+          <t>2026850002007502616</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="22" customHeight="1">
+      <c r="A141" s="6" t="inlineStr">
+        <is>
+          <t>0384045-71.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B141" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C141" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D141" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006506235</t>
+        </is>
+      </c>
+    </row>
+    <row r="142" ht="22" customHeight="1">
+      <c r="A142" s="3" t="inlineStr">
+        <is>
+          <t>0388400-27.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B142" s="4" t="inlineStr">
+        <is>
+          <t>15º VF PE</t>
+        </is>
+      </c>
+      <c r="C142" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D142" s="4" t="inlineStr">
+        <is>
+          <t>2026830000015504224</t>
+        </is>
+      </c>
+    </row>
+    <row r="143" ht="22" customHeight="1">
+      <c r="A143" s="6" t="inlineStr">
+        <is>
+          <t>0385350-90.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B143" s="7" t="inlineStr">
+        <is>
+          <t>20º VF CE</t>
+        </is>
+      </c>
+      <c r="C143" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D143" s="7" t="inlineStr">
+        <is>
+          <t>2026810000020500231</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="22" customHeight="1">
+      <c r="A144" s="3" t="inlineStr">
+        <is>
+          <t>0407941-46.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B144" s="4" t="inlineStr">
+        <is>
+          <t>6º VF PB</t>
+        </is>
+      </c>
+      <c r="C144" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D144" s="4" t="inlineStr">
+        <is>
+          <t>2026820001006502259</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="22" customHeight="1">
+      <c r="A145" s="6" t="inlineStr">
+        <is>
+          <t>0385262-52.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B145" s="7" t="inlineStr">
+        <is>
+          <t>5º VF CE</t>
+        </is>
+      </c>
+      <c r="C145" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D145" s="7" t="inlineStr">
+        <is>
+          <t>2026810000005500114</t>
+        </is>
+      </c>
+    </row>
+    <row r="146" ht="22" customHeight="1">
+      <c r="A146" s="3" t="inlineStr">
+        <is>
+          <t>0383355-42.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B146" s="4" t="inlineStr">
+        <is>
+          <t>11º VF RN</t>
+        </is>
+      </c>
+      <c r="C146" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D146" s="4" t="inlineStr">
+        <is>
+          <t>2026840003011501417</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="22" customHeight="1">
+      <c r="A147" s="6" t="inlineStr">
+        <is>
+          <t>0385353-45.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B147" s="7" t="inlineStr">
+        <is>
+          <t>5º VF CE</t>
+        </is>
+      </c>
+      <c r="C147" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D147" s="7" t="inlineStr">
+        <is>
+          <t>2026810000005500201</t>
+        </is>
+      </c>
+    </row>
+    <row r="148" ht="22" customHeight="1">
+      <c r="A148" s="3" t="inlineStr">
+        <is>
+          <t>0415223-38.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B148" s="4" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C148" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D148" s="4" t="inlineStr">
+        <is>
+          <t>2026800000014505280</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="22" customHeight="1">
+      <c r="A149" s="6" t="inlineStr">
+        <is>
+          <t>0414901-18.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B149" s="7" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C149" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D149" s="7" t="inlineStr">
+        <is>
+          <t>2026800000014504086</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="22" customHeight="1">
+      <c r="A150" s="3" t="inlineStr">
+        <is>
+          <t>0414921-09.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B150" s="4" t="inlineStr">
+        <is>
+          <t>14º VF AL</t>
+        </is>
+      </c>
+      <c r="C150" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D150" s="4" t="inlineStr">
+        <is>
+          <t>2026800000014504299</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="22" customHeight="1">
+      <c r="A151" s="6" t="inlineStr">
+        <is>
+          <t>0383925-28.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B151" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C151" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D151" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006506140</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="22" customHeight="1">
+      <c r="A152" s="3" t="inlineStr">
+        <is>
+          <t>0390869-46.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B152" s="4" t="inlineStr">
+        <is>
+          <t>3º VF RN</t>
+        </is>
+      </c>
+      <c r="C152" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D152" s="4" t="inlineStr">
+        <is>
+          <t>2026840000003502623</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="22" customHeight="1">
+      <c r="A153" s="6" t="inlineStr">
+        <is>
+          <t>0383575-40.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B153" s="7" t="inlineStr">
+        <is>
+          <t>19º VF PE</t>
+        </is>
+      </c>
+      <c r="C153" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D153" s="7" t="inlineStr">
+        <is>
+          <t>2026830000019502172</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="22" customHeight="1">
+      <c r="A154" s="3" t="inlineStr">
+        <is>
+          <t>0402478-26.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B154" s="4" t="inlineStr">
+        <is>
+          <t>2º VF CE</t>
+        </is>
+      </c>
+      <c r="C154" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D154" s="4" t="inlineStr">
+        <is>
+          <t>2026810000002500053</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="22" customHeight="1">
+      <c r="A155" s="6" t="inlineStr">
+        <is>
+          <t>0403207-52.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B155" s="7" t="inlineStr">
+        <is>
+          <t>15º VF PE</t>
+        </is>
+      </c>
+      <c r="C155" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D155" s="7" t="inlineStr">
+        <is>
+          <t>2026830000015504464</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="22" customHeight="1">
+      <c r="A156" s="3" t="inlineStr">
+        <is>
+          <t>0387887-59.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B156" s="4" t="inlineStr">
+        <is>
+          <t>10º VF RN</t>
+        </is>
+      </c>
+      <c r="C156" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D156" s="4" t="inlineStr">
+        <is>
+          <t>2026840001010500066</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="22" customHeight="1">
+      <c r="A157" s="6" t="inlineStr">
+        <is>
+          <t>0389784-25.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B157" s="7" t="inlineStr">
+        <is>
+          <t>7º VF RN</t>
+        </is>
+      </c>
+      <c r="C157" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D157" s="7" t="inlineStr">
+        <is>
+          <t>2026840000007503827</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="22" customHeight="1">
+      <c r="A158" s="3" t="inlineStr">
+        <is>
+          <t>0420128-86.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B158" s="4" t="inlineStr">
+        <is>
+          <t>29º VF PE</t>
+        </is>
+      </c>
+      <c r="C158" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D158" s="4" t="inlineStr">
+        <is>
+          <t>2026830011029501462</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="22" customHeight="1">
+      <c r="A159" s="6" t="inlineStr">
+        <is>
+          <t>0387842-55.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B159" s="7" t="inlineStr">
+        <is>
+          <t>33º VF CE</t>
+        </is>
+      </c>
+      <c r="C159" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D159" s="7" t="inlineStr">
+        <is>
+          <t>2026810000033500103</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="22" customHeight="1">
+      <c r="A160" s="3" t="inlineStr">
+        <is>
+          <t>0420069-98.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B160" s="4" t="inlineStr">
+        <is>
+          <t>20º VF CE</t>
+        </is>
+      </c>
+      <c r="C160" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D160" s="4" t="inlineStr">
+        <is>
+          <t>2026810000020500263</t>
+        </is>
+      </c>
+    </row>
+    <row r="161" ht="22" customHeight="1">
+      <c r="A161" s="6" t="inlineStr">
+        <is>
+          <t>0403221-36.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B161" s="7" t="inlineStr">
+        <is>
+          <t>20º VF CE</t>
+        </is>
+      </c>
+      <c r="C161" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D161" s="7" t="inlineStr">
+        <is>
+          <t>2026810000020500241</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="22" customHeight="1">
+      <c r="A162" s="3" t="inlineStr">
+        <is>
+          <t>0384359-17.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B162" s="4" t="inlineStr">
+        <is>
+          <t>1º VF RN</t>
+        </is>
+      </c>
+      <c r="C162" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D162" s="4" t="inlineStr">
+        <is>
+          <t>2026840000001500130</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="22" customHeight="1">
+      <c r="A163" s="6" t="inlineStr">
+        <is>
+          <t>0356828-53.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B163" s="7" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C163" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D163" s="7" t="inlineStr">
+        <is>
+          <t>2026800000009501679</t>
+        </is>
+      </c>
+    </row>
+    <row r="164" ht="22" customHeight="1">
+      <c r="A164" s="3" t="inlineStr">
+        <is>
+          <t>0382456-44.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B164" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C164" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D164" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006506009</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="22" customHeight="1">
+      <c r="A165" s="6" t="inlineStr">
+        <is>
+          <t>0362695-27.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B165" s="7" t="inlineStr">
+        <is>
+          <t>11º VF AL</t>
+        </is>
+      </c>
+      <c r="C165" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D165" s="7" t="inlineStr">
+        <is>
+          <t>2026800003011503617</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="22" customHeight="1">
+      <c r="A166" s="3" t="inlineStr">
+        <is>
+          <t>0382136-91.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B166" s="4" t="inlineStr">
+        <is>
+          <t>19º VF PE</t>
+        </is>
+      </c>
+      <c r="C166" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D166" s="4" t="inlineStr">
+        <is>
+          <t>2026830000019502052</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="22" customHeight="1">
+      <c r="A167" s="6" t="inlineStr">
+        <is>
+          <t>0382432-16.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B167" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C167" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D167" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006505985</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="22" customHeight="1">
+      <c r="A168" s="3" t="inlineStr">
+        <is>
+          <t>0359580-95.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B168" s="4" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C168" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D168" s="4" t="inlineStr">
+        <is>
+          <t>2026800000009502367</t>
+        </is>
+      </c>
+    </row>
+    <row r="169" ht="22" customHeight="1">
+      <c r="A169" s="6" t="inlineStr">
+        <is>
+          <t>0347812-75.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B169" s="7" t="inlineStr">
+        <is>
+          <t>13º VF CE</t>
+        </is>
+      </c>
+      <c r="C169" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D169" s="7" t="inlineStr">
+        <is>
+          <t>2026810000013501925</t>
+        </is>
+      </c>
+    </row>
+    <row r="170" ht="22" customHeight="1">
+      <c r="A170" s="3" t="inlineStr">
+        <is>
+          <t>0358612-65.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B170" s="4" t="inlineStr">
+        <is>
+          <t>7º VF AL</t>
+        </is>
+      </c>
+      <c r="C170" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D170" s="4" t="inlineStr">
+        <is>
+          <t>2026800002007501663</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="22" customHeight="1">
+      <c r="A171" s="6" t="inlineStr">
+        <is>
+          <t>0358613-50.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B171" s="7" t="inlineStr">
+        <is>
+          <t>7º VF AL</t>
+        </is>
+      </c>
+      <c r="C171" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D171" s="7" t="inlineStr">
+        <is>
+          <t>2026800002007501664</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="22" customHeight="1">
+      <c r="A172" s="3" t="inlineStr">
+        <is>
+          <t>0341971-02.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B172" s="4" t="inlineStr">
+        <is>
+          <t>5º VF CE</t>
+        </is>
+      </c>
+      <c r="C172" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D172" s="4" t="inlineStr">
+        <is>
+          <t>2026810000005500080</t>
+        </is>
+      </c>
+    </row>
+    <row r="173" ht="22" customHeight="1">
+      <c r="A173" s="6" t="inlineStr">
+        <is>
+          <t>0359006-72.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B173" s="7" t="inlineStr">
+        <is>
+          <t>3º VF PE</t>
+        </is>
+      </c>
+      <c r="C173" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D173" s="7" t="inlineStr">
+        <is>
+          <t>2026850000003500122</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="22" customHeight="1">
+      <c r="A174" s="3" t="inlineStr">
+        <is>
+          <t>0359223-18.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B174" s="4" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C174" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D174" s="4" t="inlineStr">
+        <is>
+          <t>2026800000009501961</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="22" customHeight="1">
+      <c r="A175" s="6" t="inlineStr">
+        <is>
+          <t>0358984-14.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B175" s="7" t="inlineStr">
+        <is>
+          <t>7º VF AL</t>
+        </is>
+      </c>
+      <c r="C175" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D175" s="7" t="inlineStr">
+        <is>
+          <t>2026800002007502057</t>
+        </is>
+      </c>
+    </row>
+    <row r="176" ht="22" customHeight="1">
+      <c r="A176" s="3" t="inlineStr">
+        <is>
+          <t>0359007-57.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B176" s="4" t="inlineStr">
+        <is>
+          <t>3º VF PE</t>
+        </is>
+      </c>
+      <c r="C176" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D176" s="4" t="inlineStr">
+        <is>
+          <t>2026850000003500124</t>
+        </is>
+      </c>
+    </row>
+    <row r="177" ht="22" customHeight="1">
+      <c r="A177" s="6" t="inlineStr">
+        <is>
+          <t>0358388-30.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B177" s="7" t="inlineStr">
+        <is>
+          <t>12º VF AL</t>
+        </is>
+      </c>
+      <c r="C177" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D177" s="7" t="inlineStr">
+        <is>
+          <t>2026800001012501762</t>
+        </is>
+      </c>
+    </row>
+    <row r="178" ht="22" customHeight="1">
+      <c r="A178" s="3" t="inlineStr">
+        <is>
+          <t>0359326-25.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B178" s="4" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C178" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D178" s="4" t="inlineStr">
+        <is>
+          <t>2026800000009502069</t>
+        </is>
+      </c>
+    </row>
+    <row r="179" ht="22" customHeight="1">
+      <c r="A179" s="6" t="inlineStr">
+        <is>
+          <t>0359466-59.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B179" s="7" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C179" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D179" s="7" t="inlineStr">
+        <is>
+          <t>2026800000009502353</t>
+        </is>
+      </c>
+    </row>
+    <row r="180" ht="22" customHeight="1">
+      <c r="A180" s="3" t="inlineStr">
+        <is>
+          <t>0359008-42.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B180" s="4" t="inlineStr">
+        <is>
+          <t>3º VF PE</t>
+        </is>
+      </c>
+      <c r="C180" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D180" s="4" t="inlineStr">
+        <is>
+          <t>2026850000003500123</t>
+        </is>
+      </c>
+    </row>
+    <row r="181" ht="22" customHeight="1">
+      <c r="A181" s="6" t="inlineStr">
+        <is>
+          <t>0348140-05.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B181" s="7" t="inlineStr">
+        <is>
+          <t>19º VF PE</t>
+        </is>
+      </c>
+      <c r="C181" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D181" s="7" t="inlineStr">
+        <is>
+          <t>2026830000019501512</t>
+        </is>
+      </c>
+    </row>
+    <row r="182" ht="22" customHeight="1">
+      <c r="A182" s="3" t="inlineStr">
+        <is>
+          <t>0373788-84.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B182" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C182" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D182" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006505790</t>
+        </is>
+      </c>
+    </row>
+    <row r="183" ht="22" customHeight="1">
+      <c r="A183" s="6" t="inlineStr">
+        <is>
+          <t>0375116-49.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B183" s="7" t="inlineStr">
+        <is>
+          <t>10º VF AL</t>
+        </is>
+      </c>
+      <c r="C183" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D183" s="7" t="inlineStr">
+        <is>
+          <t>2026800001010501951</t>
+        </is>
+      </c>
+    </row>
+    <row r="184" ht="22" customHeight="1">
+      <c r="A184" s="3" t="inlineStr">
+        <is>
+          <t>0359518-55.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B184" s="4" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C184" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D184" s="4" t="inlineStr">
+        <is>
+          <t>2026800000009502307</t>
+        </is>
+      </c>
+    </row>
+    <row r="185" ht="22" customHeight="1">
+      <c r="A185" s="6" t="inlineStr">
+        <is>
+          <t>0358334-64.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B185" s="7" t="inlineStr">
+        <is>
+          <t>12º VF AL</t>
+        </is>
+      </c>
+      <c r="C185" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D185" s="7" t="inlineStr">
+        <is>
+          <t>2026800001012501715</t>
+        </is>
+      </c>
+    </row>
+    <row r="186" ht="22" customHeight="1">
+      <c r="A186" s="3" t="inlineStr">
+        <is>
+          <t>0373803-53.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B186" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C186" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D186" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006505775</t>
+        </is>
+      </c>
+    </row>
+    <row r="187" ht="22" customHeight="1">
+      <c r="A187" s="6" t="inlineStr">
+        <is>
+          <t>0346219-11.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B187" s="7" t="inlineStr">
+        <is>
+          <t>15º VF PE</t>
+        </is>
+      </c>
+      <c r="C187" s="8" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D187" s="7" t="inlineStr">
+        <is>
+          <t>2026830000015503416</t>
+        </is>
+      </c>
+    </row>
+    <row r="188" ht="22" customHeight="1">
+      <c r="A188" s="3" t="inlineStr">
+        <is>
+          <t>0361791-07.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B188" s="4" t="inlineStr">
+        <is>
+          <t>15º VF PE</t>
+        </is>
+      </c>
+      <c r="C188" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D188" s="4" t="inlineStr">
+        <is>
+          <t>2026830000015503736</t>
+        </is>
+      </c>
+    </row>
+    <row r="189" ht="22" customHeight="1">
+      <c r="A189" s="6" t="inlineStr">
+        <is>
+          <t>0375118-19.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B189" s="7" t="inlineStr">
+        <is>
+          <t>10º VF AL</t>
+        </is>
+      </c>
+      <c r="C189" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D189" s="7" t="inlineStr">
+        <is>
+          <t>2026800001010501953</t>
+        </is>
+      </c>
+    </row>
+    <row r="190" ht="22" customHeight="1">
+      <c r="A190" s="3" t="inlineStr">
+        <is>
+          <t>0359556-67.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B190" s="4" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="C190" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D190" s="4" t="inlineStr">
+        <is>
+          <t>2026800000009502440</t>
+        </is>
+      </c>
+    </row>
+    <row r="191" ht="22" customHeight="1">
+      <c r="A191" s="6" t="inlineStr">
+        <is>
+          <t>0379231-16.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B191" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C191" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D191" s="7" t="inlineStr">
+        <is>
+          <t>2026800000006505892</t>
+        </is>
+      </c>
+    </row>
+    <row r="192" ht="22" customHeight="1">
+      <c r="A192" s="3" t="inlineStr">
+        <is>
+          <t>0373735-06.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B192" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C192" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D192" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006505803</t>
+        </is>
+      </c>
+    </row>
+    <row r="193" ht="22" customHeight="1">
+      <c r="A193" s="6" t="inlineStr">
+        <is>
+          <t>0380962-47.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B193" s="7" t="inlineStr">
+        <is>
+          <t>28º VF CE</t>
+        </is>
+      </c>
+      <c r="C193" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D193" s="7" t="inlineStr">
+        <is>
+          <t>2026810000028501612</t>
+        </is>
+      </c>
+    </row>
+    <row r="194" ht="22" customHeight="1">
+      <c r="A194" s="3" t="inlineStr">
+        <is>
+          <t>0348861-54.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B194" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C194" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D194" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006504793</t>
+        </is>
+      </c>
+    </row>
+    <row r="195" ht="22" customHeight="1">
+      <c r="A195" s="6" t="inlineStr">
+        <is>
+          <t>0372944-37.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B195" s="7" t="inlineStr">
+        <is>
+          <t>33º VF CE</t>
+        </is>
+      </c>
+      <c r="C195" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D195" s="7" t="inlineStr">
+        <is>
+          <t>2026810000033500074</t>
+        </is>
+      </c>
+    </row>
+    <row r="196" ht="22" customHeight="1">
+      <c r="A196" s="3" t="inlineStr">
+        <is>
+          <t>0342795-58.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B196" s="4" t="inlineStr">
+        <is>
+          <t>19º VF PE</t>
+        </is>
+      </c>
+      <c r="C196" s="5" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal</t>
+        </is>
+      </c>
+      <c r="D196" s="4" t="inlineStr">
+        <is>
+          <t>2026830000019500688</t>
+        </is>
+      </c>
+    </row>
+    <row r="197" ht="22" customHeight="1">
+      <c r="A197" s="6" t="inlineStr">
+        <is>
+          <t>0365537-77.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B197" s="7" t="inlineStr">
+        <is>
+          <t>4º VF SE</t>
+        </is>
+      </c>
+      <c r="C197" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D197" s="7" t="inlineStr">
+        <is>
+          <t>2026850000004500243</t>
+        </is>
+      </c>
+    </row>
+    <row r="198" ht="22" customHeight="1">
+      <c r="A198" s="3" t="inlineStr">
+        <is>
+          <t>0373697-91.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B198" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="C198" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D198" s="4" t="inlineStr">
+        <is>
+          <t>2026800000006505725</t>
+        </is>
+      </c>
+    </row>
+    <row r="199" ht="22" customHeight="1">
+      <c r="A199" s="6" t="inlineStr">
+        <is>
+          <t>0376274-42.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B199" s="7" t="inlineStr">
+        <is>
+          <t>16º VF PE</t>
+        </is>
+      </c>
+      <c r="C199" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D199" s="7" t="inlineStr">
+        <is>
+          <t>2026830002016500554</t>
+        </is>
+      </c>
+    </row>
+    <row r="200" ht="22" customHeight="1">
+      <c r="A200" s="3" t="inlineStr">
+        <is>
+          <t>0378189-29.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B200" s="4" t="inlineStr">
+        <is>
+          <t>30º VF PE</t>
+        </is>
+      </c>
+      <c r="C200" s="5" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D200" s="4" t="inlineStr">
+        <is>
+          <t>2026830011030500733</t>
+        </is>
+      </c>
+    </row>
+    <row r="201" ht="22" customHeight="1">
+      <c r="A201" s="6" t="inlineStr">
+        <is>
+          <t>0374398-52.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="B201" s="7" t="inlineStr">
+        <is>
+          <t>12º VF AL</t>
+        </is>
+      </c>
+      <c r="C201" s="8" t="inlineStr">
+        <is>
+          <t>Banco do Brasil S/A</t>
+        </is>
+      </c>
+      <c r="D201" s="7" t="inlineStr">
+        <is>
+          <t>2026800001012501981</t>
         </is>
       </c>
     </row>
@@ -2775,6 +4935,106 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A99" r:id="rId98"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A100" r:id="rId99"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A151" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A152" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A153" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A154" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A155" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A156" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A157" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A165" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A166" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A167" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A168" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A169" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A170" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A171" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A172" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A173" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A174" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A175" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A176" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A177" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A178" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A179" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A180" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A181" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A182" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A183" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A184" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A185" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A186" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A187" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A188" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A189" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A190" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A191" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A192" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A193" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A194" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A195" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A196" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A197" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A198" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A199" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A200" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A201" r:id="rId200"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
arrumar o botão de excel
</commit_message>
<xml_diff>
--- a/relatorio_rpv.xlsx
+++ b/relatorio_rpv.xlsx
@@ -7,9 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="RPV" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="RPVs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RPVs'!$A$1:$F$11</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -17,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -26,47 +28,15 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <color rgb="000056B3"/>
-      <sz val="10"/>
-      <u val="single"/>
-    </font>
-    <font>
-      <name val="Segoe UI"/>
-      <color rgb="00333333"/>
-      <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="2">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="001B365D"/>
-        <bgColor rgb="001B365D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00F8FAFC"/>
-        <bgColor rgb="00F8FAFC"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -78,48 +48,22 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color rgb="00E0E0E0"/>
-      </left>
-      <right style="thin">
-        <color rgb="00E0E0E0"/>
-      </right>
-      <top style="thin">
-        <color rgb="00E0E0E0"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00E0E0E0"/>
-      </bottom>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -486,270 +430,251 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
-    <col width="23" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="28" customHeight="1">
+    <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Nome</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Número Processo</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Proc. Originário</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Vara</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Banco</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Nº RPV</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>0459927-39.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="B2" s="4" t="inlineStr">
-        <is>
-          <t>20º VF CE</t>
-        </is>
-      </c>
-      <c r="C2" s="5" t="inlineStr">
-        <is>
-          <t>Banco do Brasil S/A</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>2026810000020500360</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="22" customHeight="1">
-      <c r="A3" s="6" t="inlineStr">
-        <is>
-          <t>0458573-76.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>13º VF PE</t>
-        </is>
-      </c>
-      <c r="C3" s="8" t="inlineStr">
-        <is>
-          <t>Banco do Brasil S/A</t>
-        </is>
-      </c>
-      <c r="D3" s="7" t="inlineStr">
-        <is>
-          <t>2026820000013510143</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="22" customHeight="1">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>0454207-91.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="B4" s="4" t="inlineStr">
-        <is>
-          <t>7º VF RN</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>Banco do Brasil S/A</t>
-        </is>
-      </c>
-      <c r="D4" s="4" t="inlineStr">
-        <is>
-          <t>2026840000007505433</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>0459281-29.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>14º VF PE</t>
-        </is>
-      </c>
-      <c r="C5" s="8" t="inlineStr">
-        <is>
-          <t>Banco do Brasil S/A</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>2026830000014504238</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>0452735-55.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="B6" s="4" t="inlineStr">
-        <is>
-          <t>14º VF AL</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>Banco do Brasil S/A</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>2026800000014508926</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>0459836-46.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>3º VF RN</t>
-        </is>
-      </c>
-      <c r="C7" s="8" t="inlineStr">
-        <is>
-          <t>Banco do Brasil S/A</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>2026840000003503607</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>0459916-10.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>20º VF CE</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>Banco do Brasil S/A</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>2026810000020500364</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>0458903-73.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>3º VF PE</t>
-        </is>
-      </c>
-      <c r="C9" s="8" t="inlineStr">
-        <is>
-          <t>Banco do Brasil S/A</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>2026820000003500707</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>0452854-16.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="inlineStr">
-        <is>
-          <t>14º VF AL</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>Banco do Brasil S/A</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>2026800000014508192</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>0459910-03.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>20º VF CE</t>
-        </is>
-      </c>
-      <c r="C11" s="8" t="inlineStr">
-        <is>
-          <t>Banco do Brasil S/A</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>2026810000020500361</t>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>30º VF PE</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal - Liberação a partir 6º dia útil próximo mês</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>RPV4317740-PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr"/>
+      <c r="B3" s="2" t="inlineStr"/>
+      <c r="C3" s="2" t="inlineStr"/>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>13º VF AL</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal - Liberação a partir 6º dia útil próximo mês</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>RPV4318464-AL</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr"/>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr"/>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal - Liberação a partir 6º dia útil próximo mês</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>RPV4319578-AL</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr"/>
+      <c r="B5" s="2" t="inlineStr"/>
+      <c r="C5" s="2" t="inlineStr"/>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal - Liberação a partir 6º dia útil próximo mês</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>RPV4319343-AL</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" s="2" t="inlineStr"/>
+      <c r="C6" s="2" t="inlineStr"/>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal - Liberação a partir 6º dia útil próximo mês</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>RPV4319792-AL</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr"/>
+      <c r="B7" s="2" t="inlineStr"/>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal - Liberação a partir 6º dia útil próximo mês</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>RPV4319230-AL</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>10º VF AL</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal - Liberação a partir 6º dia útil próximo mês</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>RPV4318322-AL</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr"/>
+      <c r="B9" s="2" t="inlineStr"/>
+      <c r="C9" s="2" t="inlineStr"/>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal - Liberação a partir 6º dia útil próximo mês</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>RPV4319592-AL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr"/>
+      <c r="B10" s="2" t="inlineStr"/>
+      <c r="C10" s="2" t="inlineStr"/>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal - Liberação a partir 6º dia útil próximo mês</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>RPV4319269-AL</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr"/>
+      <c r="B11" s="2" t="inlineStr"/>
+      <c r="C11" s="2" t="inlineStr"/>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>9º VF AL</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Caixa Econômica Federal - Liberação a partir 6º dia útil próximo mês</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>RPV4319342-AL</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A3" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId10"/>
-  </hyperlinks>
+  <autoFilter ref="A1:F11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
'V1.5', agora pode pesquisar por CPF e CNPJ
</commit_message>
<xml_diff>
--- a/relatorio_rpv.xlsx
+++ b/relatorio_rpv.xlsx
@@ -10,7 +10,7 @@
     <sheet name="RPVs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RPVs'!$A$1:$F$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RPVs'!$A$1:$F$4</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -528,54 +528,54 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>ANTONIA PEIXOTO DA SILVA</t>
+          <t>MARIA DE FATIMA ANASTACIO DOS SANTOS</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>0426618-27.2026.4.05.0000</t>
+          <t>0405314-69.2026.4.05.0000</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>00625001120254058000</t>
+          <t>00004694620254058002</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>6º VF AL</t>
+          <t>7º VF AL</t>
         </is>
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
-          <t>CEF</t>
+          <t>DO BRASIL - ANTECIPAÇÃO DO PAGAMENTO - OS VALORES ESTARÃO DISPONÍVEIS PARA SAQUE A PARTIR DO DIA 29 DESTE MÊS.</t>
         </is>
       </c>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>RPV4317011-AL</t>
+          <t>RPV4296266-AL</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>JOSE CARLOS DA SILVA</t>
+          <t>AMARO JOSE DA SILVA</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>0429144-64.2026.4.05.0000</t>
+          <t>0286668-03.2026.4.05.0000</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>00459637120244058000</t>
+          <t>00061085120254058000</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>9º VF AL</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
@@ -585,279 +585,48 @@
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>RPV4319343-AL</t>
+          <t>RPV4186717-AL</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>MARCIA NUNES DA SILVA</t>
+          <t>PEDRO SANTOS DA SILVA</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>0429070-10.2026.4.05.0000</t>
+          <t>0256833-67.2026.4.05.0000</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>00091403520234058000</t>
+          <t>00124221320254058000</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>9º VF AL</t>
+          <t>14º VF AL</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>CEF</t>
+          <t>DO BRASIL - ANTECIPAÇÃO DO PAGAMENTO - OS VALORES ESTARÃO DISPONÍVEIS PARA SAQUE A PARTIR DO DIA 30 DESTE MÊS.</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>RPV4319269-AL</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="5" t="inlineStr">
-        <is>
-          <t>MARLEIDE BARBOSA VILLAR</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>0426978-59.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>00112173720254058003</t>
-        </is>
-      </c>
-      <c r="D5" s="7" t="inlineStr">
-        <is>
-          <t>11º VF AL</t>
-        </is>
-      </c>
-      <c r="E5" s="7" t="inlineStr">
-        <is>
-          <t>CEF</t>
-        </is>
-      </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>RPV4317238-AL</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>JEDSON DA SILVA NECO</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>0429031-13.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="inlineStr">
-        <is>
-          <t>00196625320254058000</t>
-        </is>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>9º VF AL</t>
-        </is>
-      </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>CEF</t>
-        </is>
-      </c>
-      <c r="F6" s="4" t="inlineStr">
-        <is>
-          <t>RPV4319230-AL</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="5" t="inlineStr">
-        <is>
-          <t>JOSE LUIZ DA SILVA</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
-        <is>
-          <t>0429381-98.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
-        <is>
-          <t>00196426220254058000</t>
-        </is>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
-        <is>
-          <t>9º VF AL</t>
-        </is>
-      </c>
-      <c r="E7" s="7" t="inlineStr">
-        <is>
-          <t>CEF</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>RPV4319578-AL</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>QUITERIA SEVERO VALDEVINO</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>0428095-85.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>00047649520264058001</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>10º VF AL</t>
-        </is>
-      </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>CEF</t>
-        </is>
-      </c>
-      <c r="F8" s="4" t="inlineStr">
-        <is>
-          <t>RPV4318322-AL</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>FABIANA INEZ DA SILVA MARQUES</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
-        <is>
-          <t>0429143-79.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
-        <is>
-          <t>00088029020254058000</t>
-        </is>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
-        <is>
-          <t>9º VF AL</t>
-        </is>
-      </c>
-      <c r="E9" s="7" t="inlineStr">
-        <is>
-          <t>CEF</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>RPV4319342-AL</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="22" customHeight="1">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>JUNIOR DA SILVA PEREIRA</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>0427483-50.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
-        <is>
-          <t>00195809220254058300</t>
-        </is>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>30º VF PE</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>CEF</t>
-        </is>
-      </c>
-      <c r="F10" s="4" t="inlineStr">
-        <is>
-          <t>RPV4317740-PE</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
-        <is>
-          <t>JOAO THIAGO ABS NASCIMENTO</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>0428241-29.2026.4.05.0000</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
-        <is>
-          <t>08106785220224058000</t>
-        </is>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
-        <is>
-          <t>13º VF AL</t>
-        </is>
-      </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>CEF</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>RPV4318464-AL</t>
+          <t>RPV4157317-AL</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F11"/>
+  <autoFilter ref="A1:F4"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>

<commit_message>
Refinamento do codigo V1.5
</commit_message>
<xml_diff>
--- a/relatorio_rpv.xlsx
+++ b/relatorio_rpv.xlsx
@@ -10,7 +10,7 @@
     <sheet name="RPVs" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RPVs'!$A$1:$F$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'RPVs'!$A$1:$F$11</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -482,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -528,105 +528,316 @@
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>MARIA DE FATIMA ANASTACIO DOS SANTOS</t>
+          <t>MARINEIDE XAVIER DOS SANTOS</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>0405314-69.2026.4.05.0000</t>
+          <t>0484961-16.2026.4.05.0000</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>00004694620254058002</t>
+          <t>00015145720264058000</t>
         </is>
       </c>
       <c r="D2" s="4" t="inlineStr">
         <is>
-          <t>7º VF AL</t>
-        </is>
-      </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>DO BRASIL - ANTECIPAÇÃO DO PAGAMENTO - OS VALORES ESTARÃO DISPONÍVEIS PARA SAQUE A PARTIR DO DIA 29 DESTE MÊS.</t>
-        </is>
-      </c>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr"/>
       <c r="F2" s="4" t="inlineStr">
         <is>
-          <t>RPV4296266-AL</t>
+          <t>RPV4373317-AL</t>
         </is>
       </c>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
         <is>
-          <t>AMARO JOSE DA SILVA</t>
+          <t>MARIA LUZINETE DA SILVA</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>0286668-03.2026.4.05.0000</t>
+          <t>0439583-37.2026.4.05.0000</t>
         </is>
       </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
-          <t>00061085120254058000</t>
+          <t>00075735820264058001</t>
         </is>
       </c>
       <c r="D3" s="7" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
+          <t>12º VF AL</t>
         </is>
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
-          <t>CEF</t>
+          <t>DO BRASIL - ANTECIPAÇÃO DO PAGAMENTO - OS VALORES ESTARÃO DISPONÍVEIS PARA SAQUE A PARTIR DO DIA 28 DESTE MÊS.</t>
         </is>
       </c>
       <c r="F3" s="7" t="inlineStr">
         <is>
-          <t>RPV4186717-AL</t>
+          <t>RPV4328969-AL</t>
         </is>
       </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>PEDRO SANTOS DA SILVA</t>
+          <t>FERNANDA GOMES DA SILVA</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>0256833-67.2026.4.05.0000</t>
+          <t>0499770-11.2026.4.05.0000</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>00124221320254058000</t>
+          <t>00335367820254058300</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>14º VF AL</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>DO BRASIL - ANTECIPAÇÃO DO PAGAMENTO - OS VALORES ESTARÃO DISPONÍVEIS PARA SAQUE A PARTIR DO DIA 30 DESTE MÊS.</t>
-        </is>
-      </c>
+          <t>14º VF PE</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr"/>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>RPV4157317-AL</t>
+          <t>RPV4387799-PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>ELZA MARIA GOMES DE LIMA</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>0499430-67.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>00418042420254058300</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="inlineStr">
+        <is>
+          <t>14º VF PE</t>
+        </is>
+      </c>
+      <c r="E5" s="7" t="inlineStr"/>
+      <c r="F5" s="7" t="inlineStr">
+        <is>
+          <t>RPV4387460-PE</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ARISTOTELES CORREIA DE QUEIROZ NETO</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>0498425-10.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>00062968620264058201</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>10º VF PB</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr"/>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>RPV4386463-PB</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>JAILSON TELES DA SILVA</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>0498352-38.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>00060673920254058500</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>5º VF SE</t>
+        </is>
+      </c>
+      <c r="E7" s="7" t="inlineStr"/>
+      <c r="F7" s="7" t="inlineStr">
+        <is>
+          <t>RPV4386391-SE</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="22" customHeight="1">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>JULIANA MARIA CAVALCANTE RIBEIRO RAMOS</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>0434796-62.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
+        <is>
+          <t>00378898220254058100</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>33º VF CE</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>CEF</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
+        <is>
+          <t>RPV4324698-CE</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="22" customHeight="1">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>JOSEILDA MARIA DA SILVA</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>0426615-72.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>00499707220254058000</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>CEF</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>RPV4317010-AL</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>ANTONIA PEIXOTO DA SILVA</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>0426618-27.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>00625001120254058000</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>CEF</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>RPV4317011-AL</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>JUBRANT PETRUCELI</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t>0426515-20.2026.4.05.0000</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>00141379020254058000</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>6º VF AL</t>
+        </is>
+      </c>
+      <c r="E11" s="7" t="inlineStr">
+        <is>
+          <t>CEF</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr">
+        <is>
+          <t>RPV4316911-AL</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F4"/>
+  <autoFilter ref="A1:F11"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B11" r:id="rId10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup fitToHeight="0" fitToWidth="1"/>

</xml_diff>